<commit_message>
Write HSP point total into the official sheet; align row heights with the original xls (Issue #186)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFEjSwdcUNYkR6MmbgwxZn
</commit_message>
<xml_diff>
--- a/visa-case-app/docs/official/points-calculation-table_930001673.xlsx
+++ b/visa-case-app/docs/official/points-calculation-table_930001673.xlsx
@@ -8707,7 +8707,7 @@
     <tabColor indexed="45"/>
   </sheetPr>
   <dimension ref="A1:AV113"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="2.33203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="2.33203125" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col min="1" max="13" width="2.33203125" style="1" customWidth="1"/>
     <col min="14" max="14" width="2.1640625" style="1" customWidth="1"/>
@@ -8719,7 +8719,7 @@
     <col min="42" max="16384" width="2.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48">
+    <row r="1" spans="1:48" ht="12" customHeight="1">
       <c r="A1" s="42" t="s">
         <v>281</v>
       </c>
@@ -8728,11 +8728,11 @@
       </c>
       <c r="AN1" s="24"/>
     </row>
-    <row r="2" spans="1:48">
+    <row r="2" spans="1:48" ht="12" customHeight="1">
       <c r="AM2" s="24"/>
       <c r="AN2" s="24"/>
     </row>
-    <row r="4" spans="1:48" ht="17">
+    <row r="4" spans="1:48" ht="16.5" customHeight="1">
       <c r="A4" s="412" t="s">
         <v>132</v>
       </c>
@@ -8776,7 +8776,7 @@
       <c r="AM4" s="412"/>
       <c r="AN4" s="25"/>
     </row>
-    <row r="8" spans="1:48">
+    <row r="8" spans="1:48" ht="12" customHeight="1">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -8815,7 +8815,7 @@
       <c r="AJ8" s="5"/>
       <c r="AK8" s="5"/>
     </row>
-    <row r="9" spans="1:48">
+    <row r="9" spans="1:48" ht="12" customHeight="1">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -8854,7 +8854,7 @@
       <c r="AJ9" s="5"/>
       <c r="AK9" s="5"/>
     </row>
-    <row r="10" spans="1:48">
+    <row r="10" spans="1:48" ht="12" customHeight="1">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -8893,7 +8893,7 @@
       <c r="AJ10" s="5"/>
       <c r="AK10" s="5"/>
     </row>
-    <row r="11" spans="1:48" ht="15" thickBot="1">
+    <row r="11" spans="1:48" thickBot="1" ht="12.5" customHeight="1">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -8932,7 +8932,7 @@
       <c r="AJ11" s="5"/>
       <c r="AK11" s="5"/>
     </row>
-    <row r="12" spans="1:48" ht="12" customHeight="1" thickBot="1">
+    <row r="12" spans="1:48" thickBot="1" ht="12" customHeight="1">
       <c r="A12" s="322" t="s">
         <v>3</v>
       </c>
@@ -8984,7 +8984,7 @@
       <c r="AM12" s="388"/>
       <c r="AN12" s="9"/>
     </row>
-    <row r="13" spans="1:48" ht="15" thickBot="1">
+    <row r="13" spans="1:48" thickBot="1" ht="12.5" customHeight="1">
       <c r="A13" s="325"/>
       <c r="B13" s="326"/>
       <c r="C13" s="415"/>
@@ -9258,7 +9258,7 @@
       <c r="AU17" s="30"/>
       <c r="AV17" s="30"/>
     </row>
-    <row r="18" spans="1:48" ht="59.25" customHeight="1" thickBot="1">
+    <row r="18" spans="1:48" thickBot="1" ht="59.25" customHeight="1">
       <c r="A18" s="422"/>
       <c r="B18" s="423"/>
       <c r="C18" s="424"/>
@@ -9310,7 +9310,7 @@
       <c r="AU18" s="30"/>
       <c r="AV18" s="30"/>
     </row>
-    <row r="19" spans="1:48" ht="16" customHeight="1" thickBot="1">
+    <row r="19" spans="1:48" thickBot="1" ht="16" customHeight="1">
       <c r="A19" s="322" t="s">
         <v>2</v>
       </c>
@@ -9358,7 +9358,7 @@
       <c r="AM19" s="388"/>
       <c r="AN19" s="9"/>
     </row>
-    <row r="20" spans="1:48" ht="16" customHeight="1" thickBot="1">
+    <row r="20" spans="1:48" thickBot="1" ht="16" customHeight="1">
       <c r="A20" s="439"/>
       <c r="B20" s="440"/>
       <c r="C20" s="441"/>
@@ -9408,7 +9408,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:48" ht="16" customHeight="1" thickBot="1">
+    <row r="21" spans="1:48" thickBot="1" ht="16" customHeight="1">
       <c r="A21" s="439"/>
       <c r="B21" s="440"/>
       <c r="C21" s="441"/>
@@ -9458,7 +9458,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:48" ht="16" customHeight="1" thickBot="1">
+    <row r="22" spans="1:48" thickBot="1" ht="16" customHeight="1">
       <c r="A22" s="325"/>
       <c r="B22" s="326"/>
       <c r="C22" s="415"/>
@@ -9508,7 +9508,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:48" ht="16" customHeight="1" thickBot="1">
+    <row r="23" spans="1:48" thickBot="1" ht="16" customHeight="1">
       <c r="A23" s="520" t="s">
         <v>16</v>
       </c>
@@ -9562,7 +9562,7 @@
       <c r="AM23" s="388"/>
       <c r="AN23" s="9"/>
     </row>
-    <row r="24" spans="1:48" ht="16" customHeight="1" thickBot="1">
+    <row r="24" spans="1:48" thickBot="1" ht="16" customHeight="1">
       <c r="A24" s="439"/>
       <c r="B24" s="440"/>
       <c r="C24" s="441"/>
@@ -9618,7 +9618,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="1:48" ht="16" customHeight="1" thickBot="1">
+    <row r="25" spans="1:48" thickBot="1" ht="16" customHeight="1">
       <c r="A25" s="439"/>
       <c r="B25" s="440"/>
       <c r="C25" s="441"/>
@@ -9690,7 +9690,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:48" ht="16" customHeight="1" thickBot="1">
+    <row r="26" spans="1:48" thickBot="1" ht="16" customHeight="1">
       <c r="A26" s="439"/>
       <c r="B26" s="440"/>
       <c r="C26" s="441"/>
@@ -9762,7 +9762,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:48" ht="16" customHeight="1" thickBot="1">
+    <row r="27" spans="1:48" thickBot="1" ht="16" customHeight="1">
       <c r="A27" s="439"/>
       <c r="B27" s="440"/>
       <c r="C27" s="441"/>
@@ -9830,7 +9830,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:48" ht="16" customHeight="1" thickBot="1">
+    <row r="28" spans="1:48" thickBot="1" ht="16" customHeight="1">
       <c r="A28" s="439"/>
       <c r="B28" s="440"/>
       <c r="C28" s="441"/>
@@ -9898,7 +9898,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:48" ht="16" customHeight="1" thickBot="1">
+    <row r="29" spans="1:48" thickBot="1" ht="16" customHeight="1">
       <c r="A29" s="439"/>
       <c r="B29" s="440"/>
       <c r="C29" s="441"/>
@@ -9962,7 +9962,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:48" ht="16" customHeight="1" thickBot="1">
+    <row r="30" spans="1:48" thickBot="1" ht="16" customHeight="1">
       <c r="A30" s="340"/>
       <c r="B30" s="341"/>
       <c r="C30" s="523"/>
@@ -10022,7 +10022,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:48" ht="16" customHeight="1" thickBot="1">
+    <row r="31" spans="1:48" thickBot="1" ht="16" customHeight="1">
       <c r="A31" s="309" t="s">
         <v>15</v>
       </c>
@@ -10068,7 +10068,7 @@
       <c r="AM31" s="399"/>
       <c r="AN31" s="9"/>
     </row>
-    <row r="32" spans="1:48" ht="16" customHeight="1" thickBot="1">
+    <row r="32" spans="1:48" thickBot="1" ht="16" customHeight="1">
       <c r="A32" s="294"/>
       <c r="B32" s="295"/>
       <c r="C32" s="296"/>
@@ -10118,7 +10118,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:40" ht="16" customHeight="1" thickBot="1">
+    <row r="33" spans="1:40" thickBot="1" ht="16" customHeight="1">
       <c r="A33" s="294"/>
       <c r="B33" s="295"/>
       <c r="C33" s="296"/>
@@ -10168,7 +10168,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:40" ht="16" customHeight="1" thickBot="1">
+    <row r="34" spans="1:40" thickBot="1" ht="16" customHeight="1">
       <c r="A34" s="306"/>
       <c r="B34" s="307"/>
       <c r="C34" s="308"/>
@@ -10272,7 +10272,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="36" spans="1:40">
+    <row r="36" spans="1:40" ht="12" customHeight="1">
       <c r="A36" s="519"/>
       <c r="B36" s="440"/>
       <c r="C36" s="441"/>
@@ -10548,7 +10548,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="42" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A42" s="325"/>
       <c r="B42" s="326"/>
       <c r="C42" s="415"/>
@@ -10590,7 +10590,7 @@
       <c r="AM42" s="308"/>
       <c r="AN42" s="294"/>
     </row>
-    <row r="43" spans="1:40" ht="13.5" customHeight="1" thickBot="1">
+    <row r="43" spans="1:40" thickBot="1" ht="13.5" customHeight="1">
       <c r="A43" s="416" t="s">
         <v>55</v>
       </c>
@@ -10918,7 +10918,7 @@
       <c r="AM49" s="362"/>
       <c r="AN49" s="9"/>
     </row>
-    <row r="50" spans="1:40" ht="27.75" customHeight="1" thickBot="1">
+    <row r="50" spans="1:40" thickBot="1" ht="27.75" customHeight="1">
       <c r="A50" s="419"/>
       <c r="B50" s="420"/>
       <c r="C50" s="421"/>
@@ -10960,7 +10960,7 @@
       <c r="AM50" s="290"/>
       <c r="AN50" s="9"/>
     </row>
-    <row r="51" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="51" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A51" s="419"/>
       <c r="B51" s="420"/>
       <c r="C51" s="421"/>
@@ -11012,7 +11012,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="52" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A52" s="419"/>
       <c r="B52" s="420"/>
       <c r="C52" s="421"/>
@@ -11054,7 +11054,7 @@
       <c r="AM52" s="346"/>
       <c r="AN52" s="294"/>
     </row>
-    <row r="53" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="53" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A53" s="419"/>
       <c r="B53" s="420"/>
       <c r="C53" s="421"/>
@@ -11096,7 +11096,7 @@
       <c r="AM53" s="346"/>
       <c r="AN53" s="294"/>
     </row>
-    <row r="54" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="54" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A54" s="419"/>
       <c r="B54" s="420"/>
       <c r="C54" s="421"/>
@@ -11138,7 +11138,7 @@
       <c r="AM54" s="346"/>
       <c r="AN54" s="294"/>
     </row>
-    <row r="55" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="55" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A55" s="419"/>
       <c r="B55" s="420"/>
       <c r="C55" s="421"/>
@@ -11180,7 +11180,7 @@
       <c r="AM55" s="346"/>
       <c r="AN55" s="294"/>
     </row>
-    <row r="56" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="56" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A56" s="419"/>
       <c r="B56" s="420"/>
       <c r="C56" s="421"/>
@@ -11233,7 +11233,7 @@
       <c r="AM56" s="346"/>
       <c r="AN56" s="294"/>
     </row>
-    <row r="57" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="57" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A57" s="419"/>
       <c r="B57" s="420"/>
       <c r="C57" s="421"/>
@@ -11279,7 +11279,7 @@
       <c r="AM57" s="346"/>
       <c r="AN57" s="294"/>
     </row>
-    <row r="58" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="58" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A58" s="422"/>
       <c r="B58" s="423"/>
       <c r="C58" s="424"/>
@@ -11321,7 +11321,7 @@
       <c r="AM58" s="346"/>
       <c r="AN58" s="294"/>
     </row>
-    <row r="59" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="59" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A59" s="416" t="s">
         <v>156</v>
       </c>
@@ -11375,7 +11375,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="60" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A60" s="419"/>
       <c r="B60" s="420"/>
       <c r="C60" s="421"/>
@@ -11417,7 +11417,7 @@
       <c r="AM60" s="348"/>
       <c r="AN60" s="294"/>
     </row>
-    <row r="61" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="61" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A61" s="419"/>
       <c r="B61" s="420"/>
       <c r="C61" s="421"/>
@@ -11469,7 +11469,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="62" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A62" s="419"/>
       <c r="B62" s="420"/>
       <c r="C62" s="421"/>
@@ -11738,7 +11738,7 @@
       <c r="AM67" s="288"/>
       <c r="AN67" s="294"/>
     </row>
-    <row r="68" spans="1:40" ht="15" customHeight="1" thickBot="1">
+    <row r="68" spans="1:40" thickBot="1" ht="15" customHeight="1">
       <c r="A68" s="419"/>
       <c r="B68" s="420"/>
       <c r="C68" s="421"/>
@@ -11780,7 +11780,7 @@
       <c r="AM68" s="290"/>
       <c r="AN68" s="294"/>
     </row>
-    <row r="69" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="69" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A69" s="419"/>
       <c r="B69" s="420"/>
       <c r="C69" s="421"/>
@@ -11832,7 +11832,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="70" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A70" s="419"/>
       <c r="B70" s="420"/>
       <c r="C70" s="421"/>
@@ -12182,7 +12182,7 @@
       <c r="AM77" s="556"/>
       <c r="AN77" s="9"/>
     </row>
-    <row r="78" spans="1:40" ht="12" hidden="1" customHeight="1" thickBot="1">
+    <row r="78" spans="1:40" hidden="1" thickBot="1" ht="12" customHeight="1">
       <c r="A78" s="419"/>
       <c r="B78" s="420"/>
       <c r="C78" s="421"/>
@@ -12314,7 +12314,7 @@
       <c r="AM80" s="377"/>
       <c r="AN80" s="294"/>
     </row>
-    <row r="81" spans="1:40" ht="17.25" customHeight="1" thickBot="1">
+    <row r="81" spans="1:40" thickBot="1" ht="17.25" customHeight="1">
       <c r="A81" s="419"/>
       <c r="B81" s="420"/>
       <c r="C81" s="421"/>
@@ -12578,7 +12578,7 @@
       <c r="AM86" s="539"/>
       <c r="AN86" s="4"/>
     </row>
-    <row r="87" spans="1:40" ht="49.5" customHeight="1" thickBot="1">
+    <row r="87" spans="1:40" thickBot="1" ht="49.5" customHeight="1">
       <c r="A87" s="422"/>
       <c r="B87" s="423"/>
       <c r="C87" s="424"/>
@@ -12620,7 +12620,7 @@
       <c r="AM87" s="542"/>
       <c r="AN87" s="4"/>
     </row>
-    <row r="88" spans="1:40">
+    <row r="88" spans="1:40" ht="12" customHeight="1">
       <c r="AF88" s="309" t="s">
         <v>56</v>
       </c>
@@ -12630,7 +12630,7 @@
       <c r="AJ88" s="280"/>
       <c r="AK88" s="281"/>
     </row>
-    <row r="89" spans="1:40">
+    <row r="89" spans="1:40" ht="12" customHeight="1">
       <c r="AF89" s="294"/>
       <c r="AG89" s="295"/>
       <c r="AH89" s="296"/>
@@ -12638,7 +12638,7 @@
       <c r="AJ89" s="280"/>
       <c r="AK89" s="281"/>
     </row>
-    <row r="90" spans="1:40" ht="13.5" customHeight="1" thickBot="1">
+    <row r="90" spans="1:40" thickBot="1" ht="13.5" customHeight="1">
       <c r="B90" s="295"/>
       <c r="C90" s="295"/>
       <c r="D90" s="295"/>
@@ -12746,7 +12746,7 @@
       <c r="AJ94" s="4"/>
       <c r="AK94" s="4"/>
     </row>
-    <row r="95" spans="1:40">
+    <row r="95" spans="1:40" ht="12" customHeight="1">
       <c r="AF95" s="4"/>
       <c r="AG95" s="4"/>
       <c r="AH95" s="4"/>
@@ -12754,12 +12754,12 @@
       <c r="AJ95" s="4"/>
       <c r="AK95" s="4"/>
     </row>
-    <row r="96" spans="1:40">
+    <row r="96" spans="1:40" ht="13" customHeight="1">
       <c r="A96" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="97" spans="1:40">
+    <row r="97" spans="1:40" ht="13" customHeight="1">
       <c r="A97" s="197" t="s">
         <v>64</v>
       </c>
@@ -12803,7 +12803,7 @@
       <c r="AM97" s="197"/>
       <c r="AN97" s="19"/>
     </row>
-    <row r="98" spans="1:40">
+    <row r="98" spans="1:40" ht="13" customHeight="1">
       <c r="A98" s="19"/>
       <c r="B98" s="19"/>
       <c r="C98" s="19"/>
@@ -12842,7 +12842,7 @@
       <c r="AJ98" s="19"/>
       <c r="AK98" s="19"/>
     </row>
-    <row r="99" spans="1:40">
+    <row r="99" spans="1:40" ht="13" customHeight="1">
       <c r="A99" s="19"/>
       <c r="B99" s="19"/>
       <c r="C99" s="19"/>
@@ -12881,7 +12881,7 @@
       <c r="AJ99" s="19"/>
       <c r="AK99" s="19"/>
     </row>
-    <row r="101" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="101" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A101" s="20"/>
       <c r="B101" s="20" t="s">
         <v>136</v>
@@ -12933,7 +12933,7 @@
       </c>
       <c r="AN101" s="4"/>
     </row>
-    <row r="102" spans="1:40" ht="15" thickTop="1"/>
+    <row r="102" spans="1:40" thickTop="1" ht="12.5" customHeight="1"/>
     <row r="104" spans="1:40" ht="6.75" customHeight="1">
       <c r="A104" s="277"/>
       <c r="B104" s="277"/>
@@ -13016,7 +13016,7 @@
       <c r="AL105" s="277"/>
       <c r="AM105" s="277"/>
     </row>
-    <row r="106" spans="1:40">
+    <row r="106" spans="1:40" ht="12" customHeight="1">
       <c r="A106" s="277"/>
       <c r="B106" s="277"/>
       <c r="C106" s="277"/>
@@ -13057,7 +13057,7 @@
       <c r="AL106" s="277"/>
       <c r="AM106" s="277"/>
     </row>
-    <row r="107" spans="1:40">
+    <row r="107" spans="1:40" ht="12" customHeight="1">
       <c r="A107" s="277"/>
       <c r="B107" s="277"/>
       <c r="C107" s="277"/>
@@ -13098,7 +13098,7 @@
       <c r="AL107" s="277"/>
       <c r="AM107" s="277"/>
     </row>
-    <row r="108" spans="1:40">
+    <row r="108" spans="1:40" ht="12" customHeight="1">
       <c r="A108" s="277"/>
       <c r="B108" s="277"/>
       <c r="C108" s="277"/>
@@ -13139,7 +13139,7 @@
       <c r="AL108" s="277"/>
       <c r="AM108" s="277"/>
     </row>
-    <row r="109" spans="1:40">
+    <row r="109" spans="1:40" ht="12" customHeight="1">
       <c r="A109" s="277"/>
       <c r="B109" s="277"/>
       <c r="C109" s="277"/>
@@ -13180,7 +13180,7 @@
       <c r="AL109" s="277"/>
       <c r="AM109" s="277"/>
     </row>
-    <row r="110" spans="1:40">
+    <row r="110" spans="1:40" ht="12" customHeight="1">
       <c r="A110" s="277"/>
       <c r="B110" s="278"/>
       <c r="C110" s="278"/>
@@ -13221,7 +13221,7 @@
       <c r="AL110" s="278"/>
       <c r="AM110" s="278"/>
     </row>
-    <row r="111" spans="1:40">
+    <row r="111" spans="1:40" ht="12" customHeight="1">
       <c r="A111" s="278"/>
       <c r="B111" s="278"/>
       <c r="C111" s="278"/>
@@ -13262,7 +13262,7 @@
       <c r="AL111" s="278"/>
       <c r="AM111" s="278"/>
     </row>
-    <row r="112" spans="1:40">
+    <row r="112" spans="1:40" ht="12" customHeight="1">
       <c r="A112" s="278"/>
       <c r="B112" s="278"/>
       <c r="C112" s="278"/>
@@ -13303,7 +13303,7 @@
       <c r="AL112" s="278"/>
       <c r="AM112" s="278"/>
     </row>
-    <row r="113" spans="1:39">
+    <row r="113" spans="1:39" ht="12" customHeight="1">
       <c r="A113" s="278"/>
       <c r="B113" s="278"/>
       <c r="C113" s="278"/>
@@ -13595,7 +13595,7 @@
     <tabColor indexed="51"/>
   </sheetPr>
   <dimension ref="A1:AV120"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="2.33203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="2.33203125" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col min="1" max="33" width="2.33203125" style="1" customWidth="1"/>
     <col min="34" max="34" width="1.83203125" style="1" customWidth="1"/>
@@ -13605,7 +13605,7 @@
     <col min="41" max="16384" width="2.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40">
+    <row r="1" spans="1:40" ht="12" customHeight="1">
       <c r="A1" s="42" t="s">
         <v>281</v>
       </c>
@@ -13614,11 +13614,11 @@
       </c>
       <c r="AN1" s="24"/>
     </row>
-    <row r="2" spans="1:40">
+    <row r="2" spans="1:40" ht="12" customHeight="1">
       <c r="AM2" s="24"/>
       <c r="AN2" s="24"/>
     </row>
-    <row r="4" spans="1:40" ht="17">
+    <row r="4" spans="1:40" ht="16.5" customHeight="1">
       <c r="A4" s="412" t="s">
         <v>133</v>
       </c>
@@ -13663,8 +13663,8 @@
       <c r="AN4" s="25"/>
     </row>
     <row r="5" spans="1:40" ht="6" customHeight="1"/>
-    <row r="10" spans="1:40" ht="9" customHeight="1" thickBot="1"/>
-    <row r="11" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="10" spans="1:40" thickBot="1" ht="9" customHeight="1"/>
+    <row r="11" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A11" s="322" t="s">
         <v>3</v>
       </c>
@@ -13716,7 +13716,7 @@
       <c r="AM11" s="388"/>
       <c r="AN11" s="4"/>
     </row>
-    <row r="12" spans="1:40" ht="15" thickBot="1">
+    <row r="12" spans="1:40" thickBot="1" ht="12.5" customHeight="1">
       <c r="A12" s="325"/>
       <c r="B12" s="326"/>
       <c r="C12" s="415"/>
@@ -14010,7 +14010,7 @@
       <c r="AM17" s="299"/>
       <c r="AN17" s="4"/>
     </row>
-    <row r="18" spans="1:48" ht="54.75" customHeight="1" thickBot="1">
+    <row r="18" spans="1:48" thickBot="1" ht="54.75" customHeight="1">
       <c r="A18" s="422"/>
       <c r="B18" s="423"/>
       <c r="C18" s="424"/>
@@ -14062,7 +14062,7 @@
       <c r="AU18" s="30"/>
       <c r="AV18" s="30"/>
     </row>
-    <row r="19" spans="1:48" ht="15.75" customHeight="1" thickBot="1">
+    <row r="19" spans="1:48" thickBot="1" ht="15.75" customHeight="1">
       <c r="A19" s="621" t="s">
         <v>2</v>
       </c>
@@ -14110,7 +14110,7 @@
       <c r="AM19" s="560"/>
       <c r="AN19" s="4"/>
     </row>
-    <row r="20" spans="1:48" ht="15.75" customHeight="1" thickBot="1">
+    <row r="20" spans="1:48" thickBot="1" ht="15.75" customHeight="1">
       <c r="A20" s="621"/>
       <c r="B20" s="521"/>
       <c r="C20" s="522"/>
@@ -14160,7 +14160,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:48" ht="15.75" customHeight="1" thickBot="1">
+    <row r="21" spans="1:48" thickBot="1" ht="15.75" customHeight="1">
       <c r="A21" s="439"/>
       <c r="B21" s="440"/>
       <c r="C21" s="441"/>
@@ -14210,7 +14210,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:48" ht="15.75" customHeight="1" thickBot="1">
+    <row r="22" spans="1:48" thickBot="1" ht="15.75" customHeight="1">
       <c r="A22" s="439"/>
       <c r="B22" s="440"/>
       <c r="C22" s="441"/>
@@ -14260,7 +14260,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:48" ht="15.75" customHeight="1" thickBot="1">
+    <row r="23" spans="1:48" thickBot="1" ht="15.75" customHeight="1">
       <c r="A23" s="325"/>
       <c r="B23" s="326"/>
       <c r="C23" s="415"/>
@@ -14868,7 +14868,7 @@
       <c r="AM32" s="357"/>
       <c r="AN32" s="4"/>
     </row>
-    <row r="33" spans="1:40" ht="15.75" customHeight="1" thickBot="1">
+    <row r="33" spans="1:40" thickBot="1" ht="15.75" customHeight="1">
       <c r="A33" s="306"/>
       <c r="B33" s="307"/>
       <c r="C33" s="308"/>
@@ -14910,7 +14910,7 @@
       <c r="AM33" s="634"/>
       <c r="AN33" s="4"/>
     </row>
-    <row r="34" spans="1:40" ht="15.75" customHeight="1" thickBot="1">
+    <row r="34" spans="1:40" thickBot="1" ht="15.75" customHeight="1">
       <c r="A34" s="309" t="s">
         <v>15</v>
       </c>
@@ -14956,7 +14956,7 @@
       <c r="AM34" s="564"/>
       <c r="AN34" s="4"/>
     </row>
-    <row r="35" spans="1:40" ht="15.75" customHeight="1" thickBot="1">
+    <row r="35" spans="1:40" thickBot="1" ht="15.75" customHeight="1">
       <c r="A35" s="294"/>
       <c r="B35" s="295"/>
       <c r="C35" s="296"/>
@@ -15006,7 +15006,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="36" spans="1:40" ht="15.75" customHeight="1" thickBot="1">
+    <row r="36" spans="1:40" thickBot="1" ht="15.75" customHeight="1">
       <c r="A36" s="294"/>
       <c r="B36" s="295"/>
       <c r="C36" s="296"/>
@@ -15056,7 +15056,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:40" ht="15.75" customHeight="1" thickBot="1">
+    <row r="37" spans="1:40" thickBot="1" ht="15.75" customHeight="1">
       <c r="A37" s="306"/>
       <c r="B37" s="307"/>
       <c r="C37" s="308"/>
@@ -15106,7 +15106,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="38" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A38" s="518" t="s">
         <v>19</v>
       </c>
@@ -15202,7 +15202,7 @@
       <c r="AM39" s="311"/>
       <c r="AN39" s="294"/>
     </row>
-    <row r="40" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="40" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A40" s="439"/>
       <c r="B40" s="440"/>
       <c r="C40" s="441"/>
@@ -15294,7 +15294,7 @@
       <c r="AM41" s="447"/>
       <c r="AN41" s="294"/>
     </row>
-    <row r="42" spans="1:40" ht="13.5" customHeight="1" thickBot="1">
+    <row r="42" spans="1:40" thickBot="1" ht="13.5" customHeight="1">
       <c r="A42" s="439"/>
       <c r="B42" s="440"/>
       <c r="C42" s="441"/>
@@ -15386,7 +15386,7 @@
       <c r="AM43" s="311"/>
       <c r="AN43" s="294"/>
     </row>
-    <row r="44" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="44" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A44" s="439"/>
       <c r="B44" s="440"/>
       <c r="C44" s="441"/>
@@ -15436,7 +15436,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="45" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="45" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A45" s="325"/>
       <c r="B45" s="326"/>
       <c r="C45" s="415"/>
@@ -15621,7 +15621,7 @@
       <c r="AM48" s="296"/>
       <c r="AN48" s="294"/>
     </row>
-    <row r="49" spans="1:40" ht="13.5" customHeight="1" thickBot="1">
+    <row r="49" spans="1:40" thickBot="1" ht="13.5" customHeight="1">
       <c r="A49" s="306"/>
       <c r="B49" s="307"/>
       <c r="C49" s="308"/>
@@ -15663,7 +15663,7 @@
       <c r="AM49" s="308"/>
       <c r="AN49" s="294"/>
     </row>
-    <row r="50" spans="1:40" ht="13.5" customHeight="1" thickBot="1">
+    <row r="50" spans="1:40" thickBot="1" ht="13.5" customHeight="1">
       <c r="A50" s="416" t="s">
         <v>55</v>
       </c>
@@ -15753,7 +15753,7 @@
       <c r="AM51" s="566"/>
       <c r="AN51" s="294"/>
     </row>
-    <row r="52" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="52" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A52" s="419"/>
       <c r="B52" s="420"/>
       <c r="C52" s="421"/>
@@ -15847,7 +15847,7 @@
       <c r="AM53" s="447"/>
       <c r="AN53" s="294"/>
     </row>
-    <row r="54" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="54" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A54" s="419"/>
       <c r="B54" s="420"/>
       <c r="C54" s="421"/>
@@ -15941,7 +15941,7 @@
       <c r="AM55" s="447"/>
       <c r="AN55" s="294"/>
     </row>
-    <row r="56" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="56" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A56" s="419"/>
       <c r="B56" s="420"/>
       <c r="C56" s="420"/>
@@ -15990,7 +15990,7 @@
       <c r="AM56" s="569"/>
       <c r="AN56" s="9"/>
     </row>
-    <row r="57" spans="1:40" ht="27.75" customHeight="1" thickBot="1">
+    <row r="57" spans="1:40" thickBot="1" ht="27.75" customHeight="1">
       <c r="A57" s="422"/>
       <c r="B57" s="423"/>
       <c r="C57" s="423"/>
@@ -16032,7 +16032,7 @@
       <c r="AM57" s="346"/>
       <c r="AN57" s="9"/>
     </row>
-    <row r="58" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="58" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A58" s="416" t="s">
         <v>156</v>
       </c>
@@ -16086,7 +16086,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="59" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="59" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A59" s="419"/>
       <c r="B59" s="420"/>
       <c r="C59" s="421"/>
@@ -16128,7 +16128,7 @@
       <c r="AM59" s="346"/>
       <c r="AN59" s="294"/>
     </row>
-    <row r="60" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="60" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A60" s="419"/>
       <c r="B60" s="420"/>
       <c r="C60" s="421"/>
@@ -16170,7 +16170,7 @@
       <c r="AM60" s="346"/>
       <c r="AN60" s="294"/>
     </row>
-    <row r="61" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="61" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A61" s="419"/>
       <c r="B61" s="420"/>
       <c r="C61" s="421"/>
@@ -16212,7 +16212,7 @@
       <c r="AM61" s="346"/>
       <c r="AN61" s="294"/>
     </row>
-    <row r="62" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="62" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A62" s="419"/>
       <c r="B62" s="420"/>
       <c r="C62" s="421"/>
@@ -16254,7 +16254,7 @@
       <c r="AM62" s="346"/>
       <c r="AN62" s="294"/>
     </row>
-    <row r="63" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="63" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A63" s="419"/>
       <c r="B63" s="420"/>
       <c r="C63" s="421"/>
@@ -16307,7 +16307,7 @@
       <c r="AM63" s="346"/>
       <c r="AN63" s="294"/>
     </row>
-    <row r="64" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="64" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A64" s="419"/>
       <c r="B64" s="420"/>
       <c r="C64" s="421"/>
@@ -16353,7 +16353,7 @@
       <c r="AM64" s="346"/>
       <c r="AN64" s="294"/>
     </row>
-    <row r="65" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="65" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A65" s="419"/>
       <c r="B65" s="420"/>
       <c r="C65" s="421"/>
@@ -16395,7 +16395,7 @@
       <c r="AM65" s="346"/>
       <c r="AN65" s="294"/>
     </row>
-    <row r="66" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="66" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A66" s="419"/>
       <c r="B66" s="420"/>
       <c r="C66" s="421"/>
@@ -16447,7 +16447,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="67" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="67" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A67" s="419"/>
       <c r="B67" s="420"/>
       <c r="C67" s="421"/>
@@ -16489,7 +16489,7 @@
       <c r="AM67" s="346"/>
       <c r="AN67" s="294"/>
     </row>
-    <row r="68" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="68" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A68" s="419"/>
       <c r="B68" s="420"/>
       <c r="C68" s="421"/>
@@ -16541,7 +16541,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="69" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="69" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A69" s="419"/>
       <c r="B69" s="420"/>
       <c r="C69" s="421"/>
@@ -16631,7 +16631,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="71" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="71" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A71" s="419"/>
       <c r="B71" s="420"/>
       <c r="C71" s="421"/>
@@ -16815,7 +16815,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="75" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="75" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A75" s="419"/>
       <c r="B75" s="420"/>
       <c r="C75" s="421"/>
@@ -16857,7 +16857,7 @@
       <c r="AM75" s="290"/>
       <c r="AN75" s="294"/>
     </row>
-    <row r="76" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="76" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A76" s="419"/>
       <c r="B76" s="420"/>
       <c r="C76" s="421"/>
@@ -16909,7 +16909,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="77" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="77" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A77" s="419"/>
       <c r="B77" s="420"/>
       <c r="C77" s="421"/>
@@ -17261,7 +17261,7 @@
       <c r="AM84" s="556"/>
       <c r="AN84" s="294"/>
     </row>
-    <row r="85" spans="1:40" ht="12" hidden="1" customHeight="1">
+    <row r="85" spans="1:40" hidden="1" ht="12" customHeight="1">
       <c r="A85" s="419"/>
       <c r="B85" s="420"/>
       <c r="C85" s="421"/>
@@ -17393,7 +17393,7 @@
       <c r="AM87" s="377"/>
       <c r="AN87" s="294"/>
     </row>
-    <row r="88" spans="1:40" ht="17.25" customHeight="1" thickBot="1">
+    <row r="88" spans="1:40" thickBot="1" ht="17.25" customHeight="1">
       <c r="A88" s="419"/>
       <c r="B88" s="420"/>
       <c r="C88" s="421"/>
@@ -17657,7 +17657,7 @@
       <c r="AM93" s="657"/>
       <c r="AN93" s="4"/>
     </row>
-    <row r="94" spans="1:40" ht="29.25" customHeight="1" thickBot="1">
+    <row r="94" spans="1:40" thickBot="1" ht="29.25" customHeight="1">
       <c r="A94" s="419"/>
       <c r="B94" s="420"/>
       <c r="C94" s="421"/>
@@ -17699,7 +17699,7 @@
       <c r="AM94" s="660"/>
       <c r="AN94" s="4"/>
     </row>
-    <row r="95" spans="1:40" ht="26.25" customHeight="1" thickBot="1">
+    <row r="95" spans="1:40" thickBot="1" ht="26.25" customHeight="1">
       <c r="A95" s="422"/>
       <c r="B95" s="423"/>
       <c r="C95" s="424"/>
@@ -17767,7 +17767,7 @@
       <c r="AJ97" s="280"/>
       <c r="AK97" s="281"/>
     </row>
-    <row r="98" spans="1:40" ht="9" customHeight="1" thickBot="1">
+    <row r="98" spans="1:40" thickBot="1" ht="9" customHeight="1">
       <c r="AF98" s="295"/>
       <c r="AG98" s="295"/>
       <c r="AH98" s="296"/>
@@ -17956,7 +17956,7 @@
       <c r="AK106" s="19"/>
     </row>
     <row r="107" spans="1:40" ht="12" customHeight="1"/>
-    <row r="108" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="108" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A108" s="20"/>
       <c r="B108" s="20" t="s">
         <v>136</v>
@@ -18008,7 +18008,7 @@
       </c>
       <c r="AN108" s="4"/>
     </row>
-    <row r="109" spans="1:40" ht="9.75" customHeight="1" thickTop="1"/>
+    <row r="109" spans="1:40" thickTop="1" ht="9.75" customHeight="1"/>
     <row r="110" spans="1:40" ht="5.25" customHeight="1"/>
     <row r="111" spans="1:40" ht="12" customHeight="1">
       <c r="A111" s="277"/>
@@ -18051,7 +18051,7 @@
       <c r="AL111" s="277"/>
       <c r="AM111" s="277"/>
     </row>
-    <row r="112" spans="1:40">
+    <row r="112" spans="1:40" ht="12" customHeight="1">
       <c r="A112" s="277"/>
       <c r="B112" s="277"/>
       <c r="C112" s="277"/>
@@ -18092,7 +18092,7 @@
       <c r="AL112" s="277"/>
       <c r="AM112" s="277"/>
     </row>
-    <row r="113" spans="1:39">
+    <row r="113" spans="1:39" ht="12" customHeight="1">
       <c r="A113" s="277"/>
       <c r="B113" s="277"/>
       <c r="C113" s="277"/>
@@ -18133,7 +18133,7 @@
       <c r="AL113" s="277"/>
       <c r="AM113" s="277"/>
     </row>
-    <row r="114" spans="1:39">
+    <row r="114" spans="1:39" ht="12" customHeight="1">
       <c r="A114" s="277"/>
       <c r="B114" s="277"/>
       <c r="C114" s="277"/>
@@ -18174,7 +18174,7 @@
       <c r="AL114" s="277"/>
       <c r="AM114" s="277"/>
     </row>
-    <row r="115" spans="1:39">
+    <row r="115" spans="1:39" ht="12" customHeight="1">
       <c r="A115" s="277"/>
       <c r="B115" s="277"/>
       <c r="C115" s="277"/>
@@ -18215,7 +18215,7 @@
       <c r="AL115" s="277"/>
       <c r="AM115" s="277"/>
     </row>
-    <row r="116" spans="1:39">
+    <row r="116" spans="1:39" ht="12" customHeight="1">
       <c r="A116" s="277"/>
       <c r="B116" s="277"/>
       <c r="C116" s="277"/>
@@ -18297,7 +18297,7 @@
       <c r="AL117" s="278"/>
       <c r="AM117" s="278"/>
     </row>
-    <row r="118" spans="1:39">
+    <row r="118" spans="1:39" ht="12" customHeight="1">
       <c r="A118" s="278"/>
       <c r="B118" s="278"/>
       <c r="C118" s="278"/>
@@ -18338,7 +18338,7 @@
       <c r="AL118" s="278"/>
       <c r="AM118" s="278"/>
     </row>
-    <row r="119" spans="1:39">
+    <row r="119" spans="1:39" ht="12" customHeight="1">
       <c r="A119" s="278"/>
       <c r="B119" s="278"/>
       <c r="C119" s="278"/>
@@ -18379,7 +18379,7 @@
       <c r="AL119" s="278"/>
       <c r="AM119" s="278"/>
     </row>
-    <row r="120" spans="1:39">
+    <row r="120" spans="1:39" ht="12" customHeight="1">
       <c r="A120" s="278"/>
       <c r="B120" s="278"/>
       <c r="C120" s="278"/>
@@ -18764,7 +18764,7 @@
     <tabColor indexed="50"/>
   </sheetPr>
   <dimension ref="A1:AV108"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="2.33203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="2.33203125" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col min="1" max="33" width="2.33203125" style="1" customWidth="1"/>
     <col min="34" max="34" width="1.83203125" style="1" customWidth="1"/>
@@ -18774,7 +18774,7 @@
     <col min="41" max="16384" width="2.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39">
+    <row r="1" spans="1:39" ht="12" customHeight="1">
       <c r="A1" s="42" t="s">
         <v>281</v>
       </c>
@@ -18782,10 +18782,10 @@
         <v>115</v>
       </c>
     </row>
-    <row r="2" spans="1:39">
+    <row r="2" spans="1:39" ht="12" customHeight="1">
       <c r="AM2" s="24"/>
     </row>
-    <row r="4" spans="1:39" ht="17">
+    <row r="4" spans="1:39" ht="16.5" customHeight="1">
       <c r="A4" s="412" t="s">
         <v>134</v>
       </c>
@@ -18869,8 +18869,8 @@
       <c r="AL5" s="25"/>
       <c r="AM5" s="25"/>
     </row>
-    <row r="11" spans="1:39" ht="15" thickBot="1"/>
-    <row r="12" spans="1:39" ht="12" customHeight="1" thickBot="1">
+    <row r="11" spans="1:39" thickBot="1" ht="12.5" customHeight="1"/>
+    <row r="12" spans="1:39" thickBot="1" ht="12" customHeight="1">
       <c r="A12" s="322" t="s">
         <v>3</v>
       </c>
@@ -18921,7 +18921,7 @@
       </c>
       <c r="AM12" s="388"/>
     </row>
-    <row r="13" spans="1:39" ht="15" thickBot="1">
+    <row r="13" spans="1:39" thickBot="1" ht="12.5" customHeight="1">
       <c r="A13" s="325"/>
       <c r="B13" s="326"/>
       <c r="C13" s="415"/>
@@ -19154,7 +19154,7 @@
       <c r="AL17" s="297"/>
       <c r="AM17" s="299"/>
     </row>
-    <row r="18" spans="1:48" ht="53.5" customHeight="1" thickBot="1">
+    <row r="18" spans="1:48" thickBot="1" ht="53.5" customHeight="1">
       <c r="A18" s="422"/>
       <c r="B18" s="423"/>
       <c r="C18" s="424"/>
@@ -19206,7 +19206,7 @@
       <c r="AU18" s="30"/>
       <c r="AV18" s="30"/>
     </row>
-    <row r="19" spans="1:48" ht="15.75" customHeight="1" thickBot="1">
+    <row r="19" spans="1:48" thickBot="1" ht="15.75" customHeight="1">
       <c r="A19" s="322" t="s">
         <v>2</v>
       </c>
@@ -19253,7 +19253,7 @@
       </c>
       <c r="AM19" s="560"/>
     </row>
-    <row r="20" spans="1:48" ht="15.75" customHeight="1" thickBot="1">
+    <row r="20" spans="1:48" thickBot="1" ht="15.75" customHeight="1">
       <c r="A20" s="621"/>
       <c r="B20" s="521"/>
       <c r="C20" s="522"/>
@@ -19300,7 +19300,7 @@
       <c r="AL20" s="559"/>
       <c r="AM20" s="560"/>
     </row>
-    <row r="21" spans="1:48" ht="15.75" customHeight="1" thickBot="1">
+    <row r="21" spans="1:48" thickBot="1" ht="15.75" customHeight="1">
       <c r="A21" s="439"/>
       <c r="B21" s="440"/>
       <c r="C21" s="441"/>
@@ -19347,7 +19347,7 @@
       <c r="AL21" s="559"/>
       <c r="AM21" s="560"/>
     </row>
-    <row r="22" spans="1:48" ht="15.75" customHeight="1" thickBot="1">
+    <row r="22" spans="1:48" thickBot="1" ht="15.75" customHeight="1">
       <c r="A22" s="439"/>
       <c r="B22" s="440"/>
       <c r="C22" s="441"/>
@@ -19394,7 +19394,7 @@
       <c r="AL22" s="559"/>
       <c r="AM22" s="560"/>
     </row>
-    <row r="23" spans="1:48" ht="15.75" customHeight="1" thickBot="1">
+    <row r="23" spans="1:48" thickBot="1" ht="15.75" customHeight="1">
       <c r="A23" s="325"/>
       <c r="B23" s="326"/>
       <c r="C23" s="415"/>
@@ -19711,7 +19711,7 @@
       <c r="AL29" s="356"/>
       <c r="AM29" s="357"/>
     </row>
-    <row r="30" spans="1:48" ht="15.75" customHeight="1" thickBot="1">
+    <row r="30" spans="1:48" thickBot="1" ht="15.75" customHeight="1">
       <c r="A30" s="306"/>
       <c r="B30" s="307"/>
       <c r="C30" s="308"/>
@@ -19752,7 +19752,7 @@
       <c r="AL30" s="633"/>
       <c r="AM30" s="634"/>
     </row>
-    <row r="31" spans="1:48" ht="12" customHeight="1" thickBot="1">
+    <row r="31" spans="1:48" thickBot="1" ht="12" customHeight="1">
       <c r="A31" s="520" t="s">
         <v>72</v>
       </c>
@@ -19803,7 +19803,7 @@
       </c>
       <c r="AM31" s="346"/>
     </row>
-    <row r="32" spans="1:48" ht="15" thickBot="1">
+    <row r="32" spans="1:48" thickBot="1" ht="12.5" customHeight="1">
       <c r="A32" s="519"/>
       <c r="B32" s="440"/>
       <c r="C32" s="441"/>
@@ -19844,7 +19844,7 @@
       <c r="AL32" s="345"/>
       <c r="AM32" s="346"/>
     </row>
-    <row r="33" spans="1:39" ht="15" thickBot="1">
+    <row r="33" spans="1:39" thickBot="1" ht="12.5" customHeight="1">
       <c r="A33" s="439"/>
       <c r="B33" s="440"/>
       <c r="C33" s="441"/>
@@ -19891,7 +19891,7 @@
       <c r="AL33" s="345"/>
       <c r="AM33" s="346"/>
     </row>
-    <row r="34" spans="1:39" ht="15" thickBot="1">
+    <row r="34" spans="1:39" thickBot="1" ht="12.5" customHeight="1">
       <c r="A34" s="340"/>
       <c r="B34" s="341"/>
       <c r="C34" s="523"/>
@@ -19932,7 +19932,7 @@
       <c r="AL34" s="345"/>
       <c r="AM34" s="346"/>
     </row>
-    <row r="35" spans="1:39" ht="13.5" customHeight="1" thickBot="1">
+    <row r="35" spans="1:39" thickBot="1" ht="13.5" customHeight="1">
       <c r="A35" s="416" t="s">
         <v>55</v>
       </c>
@@ -20157,7 +20157,7 @@
       </c>
       <c r="AM39" s="293"/>
     </row>
-    <row r="40" spans="1:39" ht="14.25" customHeight="1" thickBot="1">
+    <row r="40" spans="1:39" thickBot="1" ht="14.25" customHeight="1">
       <c r="A40" s="419"/>
       <c r="B40" s="420"/>
       <c r="C40" s="421"/>
@@ -20247,7 +20247,7 @@
       </c>
       <c r="AM41" s="362"/>
     </row>
-    <row r="42" spans="1:39" ht="27" customHeight="1" thickBot="1">
+    <row r="42" spans="1:39" thickBot="1" ht="27" customHeight="1">
       <c r="A42" s="419"/>
       <c r="B42" s="420"/>
       <c r="C42" s="421"/>
@@ -20288,7 +20288,7 @@
       <c r="AL42" s="289"/>
       <c r="AM42" s="290"/>
     </row>
-    <row r="43" spans="1:39" ht="12" customHeight="1" thickBot="1">
+    <row r="43" spans="1:39" thickBot="1" ht="12" customHeight="1">
       <c r="A43" s="419"/>
       <c r="B43" s="420"/>
       <c r="C43" s="421"/>
@@ -20337,7 +20337,7 @@
       </c>
       <c r="AM43" s="346"/>
     </row>
-    <row r="44" spans="1:39" ht="13.5" customHeight="1" thickBot="1">
+    <row r="44" spans="1:39" thickBot="1" ht="13.5" customHeight="1">
       <c r="A44" s="419"/>
       <c r="B44" s="420"/>
       <c r="C44" s="421"/>
@@ -20378,7 +20378,7 @@
       <c r="AL44" s="345"/>
       <c r="AM44" s="346"/>
     </row>
-    <row r="45" spans="1:39" ht="13.5" customHeight="1" thickBot="1">
+    <row r="45" spans="1:39" thickBot="1" ht="13.5" customHeight="1">
       <c r="A45" s="419"/>
       <c r="B45" s="420"/>
       <c r="C45" s="421"/>
@@ -20419,7 +20419,7 @@
       <c r="AL45" s="345"/>
       <c r="AM45" s="346"/>
     </row>
-    <row r="46" spans="1:39" ht="13.5" customHeight="1" thickBot="1">
+    <row r="46" spans="1:39" thickBot="1" ht="13.5" customHeight="1">
       <c r="A46" s="419"/>
       <c r="B46" s="420"/>
       <c r="C46" s="421"/>
@@ -20460,7 +20460,7 @@
       <c r="AL46" s="345"/>
       <c r="AM46" s="346"/>
     </row>
-    <row r="47" spans="1:39" ht="13.5" customHeight="1" thickBot="1">
+    <row r="47" spans="1:39" thickBot="1" ht="13.5" customHeight="1">
       <c r="A47" s="419"/>
       <c r="B47" s="420"/>
       <c r="C47" s="421"/>
@@ -20501,7 +20501,7 @@
       <c r="AL47" s="345"/>
       <c r="AM47" s="346"/>
     </row>
-    <row r="48" spans="1:39" ht="13.5" customHeight="1" thickBot="1">
+    <row r="48" spans="1:39" thickBot="1" ht="13.5" customHeight="1">
       <c r="A48" s="419"/>
       <c r="B48" s="420"/>
       <c r="C48" s="421"/>
@@ -20553,7 +20553,7 @@
       <c r="AL48" s="345"/>
       <c r="AM48" s="346"/>
     </row>
-    <row r="49" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="49" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A49" s="419"/>
       <c r="B49" s="420"/>
       <c r="C49" s="421"/>
@@ -20598,7 +20598,7 @@
       <c r="AL49" s="345"/>
       <c r="AM49" s="346"/>
     </row>
-    <row r="50" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="50" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A50" s="419"/>
       <c r="B50" s="420"/>
       <c r="C50" s="421"/>
@@ -20639,7 +20639,7 @@
       <c r="AL50" s="345"/>
       <c r="AM50" s="346"/>
     </row>
-    <row r="51" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="51" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A51" s="419"/>
       <c r="B51" s="420"/>
       <c r="C51" s="421"/>
@@ -20688,7 +20688,7 @@
       </c>
       <c r="AM51" s="346"/>
     </row>
-    <row r="52" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="52" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A52" s="419"/>
       <c r="B52" s="420"/>
       <c r="C52" s="421"/>
@@ -20729,7 +20729,7 @@
       <c r="AL52" s="345"/>
       <c r="AM52" s="346"/>
     </row>
-    <row r="53" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="53" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A53" s="419"/>
       <c r="B53" s="420"/>
       <c r="C53" s="421"/>
@@ -20778,7 +20778,7 @@
       </c>
       <c r="AM53" s="346"/>
     </row>
-    <row r="54" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="54" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A54" s="422"/>
       <c r="B54" s="423"/>
       <c r="C54" s="424"/>
@@ -20867,7 +20867,7 @@
       <c r="AM55" s="286"/>
       <c r="AN55" s="26"/>
     </row>
-    <row r="56" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="56" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A56" s="420"/>
       <c r="B56" s="420"/>
       <c r="C56" s="421"/>
@@ -21043,7 +21043,7 @@
       <c r="AL59" s="287"/>
       <c r="AM59" s="288"/>
     </row>
-    <row r="60" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="60" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A60" s="420"/>
       <c r="B60" s="420"/>
       <c r="C60" s="421"/>
@@ -21084,7 +21084,7 @@
       <c r="AL60" s="289"/>
       <c r="AM60" s="290"/>
     </row>
-    <row r="61" spans="1:40" ht="14.25" customHeight="1" thickBot="1">
+    <row r="61" spans="1:40" thickBot="1" ht="14.25" customHeight="1">
       <c r="A61" s="420"/>
       <c r="B61" s="420"/>
       <c r="C61" s="421"/>
@@ -21133,7 +21133,7 @@
       </c>
       <c r="AM61" s="348"/>
     </row>
-    <row r="62" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="62" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A62" s="420"/>
       <c r="B62" s="420"/>
       <c r="C62" s="421"/>
@@ -21605,7 +21605,7 @@
       <c r="AM72" s="377"/>
       <c r="AN72" s="294"/>
     </row>
-    <row r="73" spans="1:40" ht="18" customHeight="1" thickBot="1">
+    <row r="73" spans="1:40" thickBot="1" ht="18" customHeight="1">
       <c r="A73" s="420"/>
       <c r="B73" s="420"/>
       <c r="C73" s="421"/>
@@ -21647,7 +21647,7 @@
       <c r="AM73" s="380"/>
       <c r="AN73" s="294"/>
     </row>
-    <row r="74" spans="1:40" ht="16" customHeight="1" thickBot="1">
+    <row r="74" spans="1:40" thickBot="1" ht="16" customHeight="1">
       <c r="A74" s="420"/>
       <c r="B74" s="420"/>
       <c r="C74" s="421"/>
@@ -21865,7 +21865,7 @@
       <c r="AM78" s="374"/>
       <c r="AN78" s="4"/>
     </row>
-    <row r="79" spans="1:40" ht="38.25" customHeight="1" thickBot="1">
+    <row r="79" spans="1:40" thickBot="1" ht="38.25" customHeight="1">
       <c r="A79" s="420"/>
       <c r="B79" s="420"/>
       <c r="C79" s="421"/>
@@ -21907,7 +21907,7 @@
       <c r="AM79" s="634"/>
       <c r="AN79" s="4"/>
     </row>
-    <row r="80" spans="1:40" ht="21" customHeight="1" thickBot="1">
+    <row r="80" spans="1:40" thickBot="1" ht="21" customHeight="1">
       <c r="A80" s="420"/>
       <c r="B80" s="420"/>
       <c r="C80" s="421"/>
@@ -21956,7 +21956,7 @@
       </c>
       <c r="AM80" s="346"/>
     </row>
-    <row r="81" spans="1:40" ht="21" customHeight="1" thickBot="1">
+    <row r="81" spans="1:40" thickBot="1" ht="21" customHeight="1">
       <c r="A81" s="423"/>
       <c r="B81" s="423"/>
       <c r="C81" s="424"/>
@@ -22005,7 +22005,7 @@
       </c>
       <c r="AM81" s="346"/>
     </row>
-    <row r="82" spans="1:40">
+    <row r="82" spans="1:40" ht="12" customHeight="1">
       <c r="AF82" s="295" t="s">
         <v>56</v>
       </c>
@@ -22015,7 +22015,7 @@
       <c r="AJ82" s="482"/>
       <c r="AK82" s="483"/>
     </row>
-    <row r="83" spans="1:40">
+    <row r="83" spans="1:40" ht="12" customHeight="1">
       <c r="AF83" s="295"/>
       <c r="AG83" s="295"/>
       <c r="AH83" s="295"/>
@@ -22023,7 +22023,7 @@
       <c r="AJ83" s="280"/>
       <c r="AK83" s="281"/>
     </row>
-    <row r="84" spans="1:40" ht="15" thickBot="1">
+    <row r="84" spans="1:40" thickBot="1" ht="12.5" customHeight="1">
       <c r="AF84" s="295"/>
       <c r="AG84" s="295"/>
       <c r="AH84" s="295"/>
@@ -22117,7 +22117,7 @@
       <c r="AJ88" s="4"/>
       <c r="AK88" s="4"/>
     </row>
-    <row r="89" spans="1:40">
+    <row r="89" spans="1:40" ht="12" customHeight="1">
       <c r="AF89" s="4"/>
       <c r="AG89" s="4"/>
       <c r="AH89" s="4"/>
@@ -22125,12 +22125,12 @@
       <c r="AJ89" s="4"/>
       <c r="AK89" s="4"/>
     </row>
-    <row r="90" spans="1:40">
+    <row r="90" spans="1:40" ht="13" customHeight="1">
       <c r="A90" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="91" spans="1:40">
+    <row r="91" spans="1:40" ht="13" customHeight="1">
       <c r="A91" s="197" t="s">
         <v>64</v>
       </c>
@@ -22173,7 +22173,7 @@
       <c r="AL91" s="197"/>
       <c r="AM91" s="197"/>
     </row>
-    <row r="92" spans="1:40">
+    <row r="92" spans="1:40" ht="13" customHeight="1">
       <c r="A92" s="19"/>
       <c r="B92" s="19"/>
       <c r="C92" s="19"/>
@@ -22212,7 +22212,7 @@
       <c r="AJ92" s="19"/>
       <c r="AK92" s="19"/>
     </row>
-    <row r="93" spans="1:40">
+    <row r="93" spans="1:40" ht="13" customHeight="1">
       <c r="A93" s="19"/>
       <c r="B93" s="19"/>
       <c r="C93" s="19"/>
@@ -22251,7 +22251,7 @@
       <c r="AJ93" s="19"/>
       <c r="AK93" s="19"/>
     </row>
-    <row r="94" spans="1:40">
+    <row r="94" spans="1:40" ht="13" customHeight="1">
       <c r="A94" s="19"/>
       <c r="B94" s="19"/>
       <c r="C94" s="19"/>
@@ -22290,7 +22290,7 @@
       <c r="AJ94" s="19"/>
       <c r="AK94" s="19"/>
     </row>
-    <row r="96" spans="1:40" ht="12" customHeight="1" thickBot="1">
+    <row r="96" spans="1:40" thickBot="1" ht="12" customHeight="1">
       <c r="A96" s="20"/>
       <c r="B96" s="20" t="s">
         <v>136</v>
@@ -22342,7 +22342,7 @@
       </c>
       <c r="AN96" s="4"/>
     </row>
-    <row r="97" spans="1:39" ht="15" thickTop="1"/>
+    <row r="97" spans="1:39" thickTop="1" ht="12.5" customHeight="1"/>
     <row r="98" spans="1:39" ht="5.25" customHeight="1"/>
     <row r="99" spans="1:39" ht="5.25" customHeight="1">
       <c r="A99" s="277"/>
@@ -22385,7 +22385,7 @@
       <c r="AL99" s="277"/>
       <c r="AM99" s="277"/>
     </row>
-    <row r="100" spans="1:39">
+    <row r="100" spans="1:39" ht="12" customHeight="1">
       <c r="A100" s="277"/>
       <c r="B100" s="277"/>
       <c r="C100" s="277"/>
@@ -22426,7 +22426,7 @@
       <c r="AL100" s="277"/>
       <c r="AM100" s="277"/>
     </row>
-    <row r="101" spans="1:39">
+    <row r="101" spans="1:39" ht="12" customHeight="1">
       <c r="A101" s="277"/>
       <c r="B101" s="277"/>
       <c r="C101" s="277"/>
@@ -22467,7 +22467,7 @@
       <c r="AL101" s="277"/>
       <c r="AM101" s="277"/>
     </row>
-    <row r="102" spans="1:39">
+    <row r="102" spans="1:39" ht="12" customHeight="1">
       <c r="A102" s="277"/>
       <c r="B102" s="277"/>
       <c r="C102" s="277"/>
@@ -22508,7 +22508,7 @@
       <c r="AL102" s="277"/>
       <c r="AM102" s="277"/>
     </row>
-    <row r="103" spans="1:39">
+    <row r="103" spans="1:39" ht="12" customHeight="1">
       <c r="A103" s="277"/>
       <c r="B103" s="277"/>
       <c r="C103" s="277"/>
@@ -22549,7 +22549,7 @@
       <c r="AL103" s="277"/>
       <c r="AM103" s="277"/>
     </row>
-    <row r="104" spans="1:39">
+    <row r="104" spans="1:39" ht="12" customHeight="1">
       <c r="A104" s="277"/>
       <c r="B104" s="277"/>
       <c r="C104" s="277"/>
@@ -22631,7 +22631,7 @@
       <c r="AL105" s="278"/>
       <c r="AM105" s="278"/>
     </row>
-    <row r="106" spans="1:39">
+    <row r="106" spans="1:39" ht="12" customHeight="1">
       <c r="A106" s="278"/>
       <c r="B106" s="278"/>
       <c r="C106" s="278"/>
@@ -22672,7 +22672,7 @@
       <c r="AL106" s="278"/>
       <c r="AM106" s="278"/>
     </row>
-    <row r="107" spans="1:39">
+    <row r="107" spans="1:39" ht="12" customHeight="1">
       <c r="A107" s="278"/>
       <c r="B107" s="278"/>
       <c r="C107" s="278"/>
@@ -22713,7 +22713,7 @@
       <c r="AL107" s="278"/>
       <c r="AM107" s="278"/>
     </row>
-    <row r="108" spans="1:39">
+    <row r="108" spans="1:39" ht="12" customHeight="1">
       <c r="A108" s="278"/>
       <c r="B108" s="278"/>
       <c r="C108" s="278"/>
@@ -22939,19 +22939,19 @@
     <tabColor indexed="29"/>
   </sheetPr>
   <dimension ref="A1:AR152"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="2.33203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="2.33203125" defaultRowHeight="13" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="2.33203125" customWidth="1"/>
     <col min="3" max="3" width="2.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44">
+    <row r="1" spans="1:44" ht="13" customHeight="1">
       <c r="A1" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="2" spans="1:44" ht="15" thickBot="1"/>
-    <row r="3" spans="1:44">
+    <row r="2" spans="1:44" thickBot="1" ht="13.5" customHeight="1"/>
+    <row r="3" spans="1:44" ht="13" customHeight="1">
       <c r="A3" s="186" t="s">
         <v>86</v>
       </c>
@@ -23003,7 +23003,7 @@
       <c r="AQ3" s="171"/>
       <c r="AR3" s="171"/>
     </row>
-    <row r="4" spans="1:44" ht="15" thickBot="1">
+    <row r="4" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A4" s="187"/>
       <c r="B4" s="187"/>
       <c r="C4" s="187"/>
@@ -23193,7 +23193,7 @@
       <c r="AQ7" s="169"/>
       <c r="AR7" s="170"/>
     </row>
-    <row r="8" spans="1:44">
+    <row r="8" spans="1:44" ht="13" customHeight="1">
       <c r="A8" s="189"/>
       <c r="B8" s="169"/>
       <c r="C8" s="169"/>
@@ -23239,7 +23239,7 @@
       <c r="AQ8" s="169"/>
       <c r="AR8" s="170"/>
     </row>
-    <row r="9" spans="1:44" ht="15" thickBot="1">
+    <row r="9" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A9" s="151"/>
       <c r="B9" s="152"/>
       <c r="C9" s="152"/>
@@ -23285,7 +23285,7 @@
       <c r="AQ9" s="152"/>
       <c r="AR9" s="153"/>
     </row>
-    <row r="10" spans="1:44">
+    <row r="10" spans="1:44" ht="13" customHeight="1">
       <c r="A10" s="188" t="s">
         <v>177</v>
       </c>
@@ -23337,7 +23337,7 @@
       <c r="AQ10" s="166"/>
       <c r="AR10" s="167"/>
     </row>
-    <row r="11" spans="1:44">
+    <row r="11" spans="1:44" ht="13" customHeight="1">
       <c r="A11" s="151"/>
       <c r="B11" s="152"/>
       <c r="C11" s="152"/>
@@ -23383,7 +23383,7 @@
       <c r="AQ11" s="152"/>
       <c r="AR11" s="153"/>
     </row>
-    <row r="12" spans="1:44" ht="15" thickBot="1">
+    <row r="12" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A12" s="154"/>
       <c r="B12" s="155"/>
       <c r="C12" s="155"/>
@@ -23481,7 +23481,7 @@
       <c r="AQ13" s="106"/>
       <c r="AR13" s="107"/>
     </row>
-    <row r="14" spans="1:44">
+    <row r="14" spans="1:44" ht="13" customHeight="1">
       <c r="A14" s="102"/>
       <c r="B14" s="103"/>
       <c r="C14" s="103"/>
@@ -23527,7 +23527,7 @@
       <c r="AQ14" s="109"/>
       <c r="AR14" s="110"/>
     </row>
-    <row r="15" spans="1:44">
+    <row r="15" spans="1:44" ht="13" customHeight="1">
       <c r="A15" s="102"/>
       <c r="B15" s="103"/>
       <c r="C15" s="103"/>
@@ -23573,7 +23573,7 @@
       <c r="AQ15" s="109"/>
       <c r="AR15" s="110"/>
     </row>
-    <row r="16" spans="1:44">
+    <row r="16" spans="1:44" ht="13" customHeight="1">
       <c r="A16" s="102"/>
       <c r="B16" s="103"/>
       <c r="C16" s="103"/>
@@ -23621,7 +23621,7 @@
       <c r="AQ16" s="109"/>
       <c r="AR16" s="110"/>
     </row>
-    <row r="17" spans="1:44">
+    <row r="17" spans="1:44" ht="13" customHeight="1">
       <c r="A17" s="102"/>
       <c r="B17" s="103"/>
       <c r="C17" s="103"/>
@@ -23667,7 +23667,7 @@
       <c r="AQ17" s="109"/>
       <c r="AR17" s="110"/>
     </row>
-    <row r="18" spans="1:44">
+    <row r="18" spans="1:44" ht="13" customHeight="1">
       <c r="A18" s="102"/>
       <c r="B18" s="103"/>
       <c r="C18" s="103"/>
@@ -23713,7 +23713,7 @@
       <c r="AQ18" s="109"/>
       <c r="AR18" s="110"/>
     </row>
-    <row r="19" spans="1:44" ht="15" thickBot="1">
+    <row r="19" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A19" s="117"/>
       <c r="B19" s="118"/>
       <c r="C19" s="118"/>
@@ -23859,7 +23859,7 @@
       <c r="AQ21" s="152"/>
       <c r="AR21" s="153"/>
     </row>
-    <row r="22" spans="1:44">
+    <row r="22" spans="1:44" ht="13" customHeight="1">
       <c r="A22" s="151"/>
       <c r="B22" s="152"/>
       <c r="C22" s="152"/>
@@ -23957,7 +23957,7 @@
       <c r="AQ23" s="152"/>
       <c r="AR23" s="153"/>
     </row>
-    <row r="24" spans="1:44">
+    <row r="24" spans="1:44" ht="13" customHeight="1">
       <c r="A24" s="151"/>
       <c r="B24" s="152"/>
       <c r="C24" s="152"/>
@@ -24003,7 +24003,7 @@
       <c r="AQ24" s="152"/>
       <c r="AR24" s="153"/>
     </row>
-    <row r="25" spans="1:44">
+    <row r="25" spans="1:44" ht="13" customHeight="1">
       <c r="A25" s="151"/>
       <c r="B25" s="152"/>
       <c r="C25" s="152"/>
@@ -24049,7 +24049,7 @@
       <c r="AQ25" s="152"/>
       <c r="AR25" s="153"/>
     </row>
-    <row r="26" spans="1:44">
+    <row r="26" spans="1:44" ht="13" customHeight="1">
       <c r="A26" s="151"/>
       <c r="B26" s="152"/>
       <c r="C26" s="152"/>
@@ -24333,7 +24333,7 @@
       <c r="AQ31" s="152"/>
       <c r="AR31" s="153"/>
     </row>
-    <row r="32" spans="1:44">
+    <row r="32" spans="1:44" ht="13" customHeight="1">
       <c r="A32" s="102"/>
       <c r="B32" s="103"/>
       <c r="C32" s="103"/>
@@ -24379,7 +24379,7 @@
       <c r="AQ32" s="152"/>
       <c r="AR32" s="153"/>
     </row>
-    <row r="33" spans="1:44">
+    <row r="33" spans="1:44" ht="13" customHeight="1">
       <c r="A33" s="102"/>
       <c r="B33" s="103"/>
       <c r="C33" s="103"/>
@@ -24425,7 +24425,7 @@
       <c r="AQ33" s="152"/>
       <c r="AR33" s="153"/>
     </row>
-    <row r="34" spans="1:44">
+    <row r="34" spans="1:44" ht="13" customHeight="1">
       <c r="A34" s="102"/>
       <c r="B34" s="103"/>
       <c r="C34" s="103"/>
@@ -24471,7 +24471,7 @@
       <c r="AQ34" s="152"/>
       <c r="AR34" s="153"/>
     </row>
-    <row r="35" spans="1:44">
+    <row r="35" spans="1:44" ht="13" customHeight="1">
       <c r="A35" s="102"/>
       <c r="B35" s="103"/>
       <c r="C35" s="103"/>
@@ -24517,7 +24517,7 @@
       <c r="AQ35" s="152"/>
       <c r="AR35" s="153"/>
     </row>
-    <row r="36" spans="1:44">
+    <row r="36" spans="1:44" ht="13" customHeight="1">
       <c r="A36" s="102"/>
       <c r="B36" s="103"/>
       <c r="C36" s="103"/>
@@ -24563,7 +24563,7 @@
       <c r="AQ36" s="152"/>
       <c r="AR36" s="153"/>
     </row>
-    <row r="37" spans="1:44">
+    <row r="37" spans="1:44" ht="13" customHeight="1">
       <c r="A37" s="102"/>
       <c r="B37" s="103"/>
       <c r="C37" s="103"/>
@@ -24609,7 +24609,7 @@
       <c r="AQ37" s="152"/>
       <c r="AR37" s="153"/>
     </row>
-    <row r="38" spans="1:44">
+    <row r="38" spans="1:44" ht="13" customHeight="1">
       <c r="A38" s="126"/>
       <c r="B38" s="127"/>
       <c r="C38" s="127"/>
@@ -24707,7 +24707,7 @@
       <c r="AQ39" s="152"/>
       <c r="AR39" s="153"/>
     </row>
-    <row r="40" spans="1:44">
+    <row r="40" spans="1:44" ht="13" customHeight="1">
       <c r="A40" s="151"/>
       <c r="B40" s="152"/>
       <c r="C40" s="152"/>
@@ -24753,7 +24753,7 @@
       <c r="AQ40" s="152"/>
       <c r="AR40" s="153"/>
     </row>
-    <row r="41" spans="1:44" ht="15" thickBot="1">
+    <row r="41" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A41" s="154"/>
       <c r="B41" s="155"/>
       <c r="C41" s="155"/>
@@ -24799,7 +24799,7 @@
       <c r="AQ41" s="155"/>
       <c r="AR41" s="156"/>
     </row>
-    <row r="42" spans="1:44">
+    <row r="42" spans="1:44" ht="13" customHeight="1">
       <c r="A42" s="43"/>
       <c r="B42" s="38"/>
       <c r="C42" s="38"/>
@@ -24899,7 +24899,7 @@
       <c r="AQ43" s="109"/>
       <c r="AR43" s="110"/>
     </row>
-    <row r="44" spans="1:44">
+    <row r="44" spans="1:44" ht="13" customHeight="1">
       <c r="A44" s="102"/>
       <c r="B44" s="103"/>
       <c r="C44" s="103"/>
@@ -24945,7 +24945,7 @@
       <c r="AQ44" s="109"/>
       <c r="AR44" s="110"/>
     </row>
-    <row r="45" spans="1:44">
+    <row r="45" spans="1:44" ht="13" customHeight="1">
       <c r="A45" s="102"/>
       <c r="B45" s="103"/>
       <c r="C45" s="103"/>
@@ -24991,7 +24991,7 @@
       <c r="AQ45" s="109"/>
       <c r="AR45" s="110"/>
     </row>
-    <row r="46" spans="1:44">
+    <row r="46" spans="1:44" ht="13" customHeight="1">
       <c r="A46" s="102"/>
       <c r="B46" s="103"/>
       <c r="C46" s="103"/>
@@ -25037,7 +25037,7 @@
       <c r="AQ46" s="109"/>
       <c r="AR46" s="110"/>
     </row>
-    <row r="47" spans="1:44">
+    <row r="47" spans="1:44" ht="13" customHeight="1">
       <c r="A47" s="102"/>
       <c r="B47" s="103"/>
       <c r="C47" s="103"/>
@@ -25083,7 +25083,7 @@
       <c r="AQ47" s="109"/>
       <c r="AR47" s="110"/>
     </row>
-    <row r="48" spans="1:44" ht="15" thickBot="1">
+    <row r="48" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A48" s="43"/>
       <c r="B48" s="38"/>
       <c r="C48" s="38"/>
@@ -25413,7 +25413,7 @@
       <c r="AQ54" s="109"/>
       <c r="AR54" s="110"/>
     </row>
-    <row r="55" spans="1:44">
+    <row r="55" spans="1:44" ht="13" customHeight="1">
       <c r="A55" s="102"/>
       <c r="B55" s="103"/>
       <c r="C55" s="103"/>
@@ -25459,7 +25459,7 @@
       <c r="AQ55" s="109"/>
       <c r="AR55" s="110"/>
     </row>
-    <row r="56" spans="1:44">
+    <row r="56" spans="1:44" ht="13" customHeight="1">
       <c r="A56" s="102"/>
       <c r="B56" s="103"/>
       <c r="C56" s="103"/>
@@ -25505,7 +25505,7 @@
       <c r="AQ56" s="109"/>
       <c r="AR56" s="110"/>
     </row>
-    <row r="57" spans="1:44">
+    <row r="57" spans="1:44" ht="13" customHeight="1">
       <c r="A57" s="102"/>
       <c r="B57" s="103"/>
       <c r="C57" s="103"/>
@@ -25551,7 +25551,7 @@
       <c r="AQ57" s="109"/>
       <c r="AR57" s="110"/>
     </row>
-    <row r="58" spans="1:44" ht="15" thickBot="1">
+    <row r="58" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A58" s="117"/>
       <c r="B58" s="118"/>
       <c r="C58" s="118"/>
@@ -25973,7 +25973,7 @@
       <c r="AQ66" s="109"/>
       <c r="AR66" s="110"/>
     </row>
-    <row r="67" spans="1:44">
+    <row r="67" spans="1:44" ht="13" customHeight="1">
       <c r="A67" s="102"/>
       <c r="B67" s="103"/>
       <c r="C67" s="103"/>
@@ -26019,7 +26019,7 @@
       <c r="AQ67" s="109"/>
       <c r="AR67" s="110"/>
     </row>
-    <row r="68" spans="1:44">
+    <row r="68" spans="1:44" ht="13" customHeight="1">
       <c r="A68" s="102"/>
       <c r="B68" s="103"/>
       <c r="C68" s="103"/>
@@ -26111,7 +26111,7 @@
       <c r="AQ69" s="109"/>
       <c r="AR69" s="110"/>
     </row>
-    <row r="70" spans="1:44" ht="15" thickBot="1">
+    <row r="70" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A70" s="117"/>
       <c r="B70" s="118"/>
       <c r="C70" s="118"/>
@@ -26157,7 +26157,7 @@
       <c r="AQ70" s="109"/>
       <c r="AR70" s="110"/>
     </row>
-    <row r="71" spans="1:44">
+    <row r="71" spans="1:44" ht="13" customHeight="1">
       <c r="A71" s="133" t="s">
         <v>218</v>
       </c>
@@ -26255,7 +26255,7 @@
       <c r="AQ72" s="109"/>
       <c r="AR72" s="110"/>
     </row>
-    <row r="73" spans="1:44">
+    <row r="73" spans="1:44" ht="13" customHeight="1">
       <c r="A73" s="136"/>
       <c r="B73" s="137"/>
       <c r="C73" s="137"/>
@@ -26301,7 +26301,7 @@
       <c r="AQ73" s="109"/>
       <c r="AR73" s="110"/>
     </row>
-    <row r="74" spans="1:44" ht="36.75" customHeight="1" thickBot="1">
+    <row r="74" spans="1:44" thickBot="1" ht="36.75" customHeight="1">
       <c r="A74" s="139"/>
       <c r="B74" s="140"/>
       <c r="C74" s="140"/>
@@ -26347,7 +26347,7 @@
       <c r="AQ74" s="109"/>
       <c r="AR74" s="110"/>
     </row>
-    <row r="75" spans="1:44">
+    <row r="75" spans="1:44" ht="13" customHeight="1">
       <c r="A75" s="99" t="s">
         <v>217</v>
       </c>
@@ -26629,7 +26629,7 @@
       <c r="AQ80" s="109"/>
       <c r="AR80" s="110"/>
     </row>
-    <row r="81" spans="1:44">
+    <row r="81" spans="1:44" ht="13" customHeight="1">
       <c r="A81" s="102"/>
       <c r="B81" s="103"/>
       <c r="C81" s="103"/>
@@ -26721,7 +26721,7 @@
       <c r="AQ82" s="109"/>
       <c r="AR82" s="110"/>
     </row>
-    <row r="83" spans="1:44">
+    <row r="83" spans="1:44" ht="13" customHeight="1">
       <c r="A83" s="102"/>
       <c r="B83" s="103"/>
       <c r="C83" s="103"/>
@@ -26767,7 +26767,7 @@
       <c r="AQ83" s="109"/>
       <c r="AR83" s="110"/>
     </row>
-    <row r="84" spans="1:44">
+    <row r="84" spans="1:44" ht="13" customHeight="1">
       <c r="A84" s="102"/>
       <c r="B84" s="103"/>
       <c r="C84" s="103"/>
@@ -26813,7 +26813,7 @@
       <c r="AQ84" s="109"/>
       <c r="AR84" s="110"/>
     </row>
-    <row r="85" spans="1:44">
+    <row r="85" spans="1:44" ht="13" customHeight="1">
       <c r="A85" s="102"/>
       <c r="B85" s="103"/>
       <c r="C85" s="103"/>
@@ -27233,7 +27233,7 @@
       <c r="AQ93" s="109"/>
       <c r="AR93" s="110"/>
     </row>
-    <row r="94" spans="1:44">
+    <row r="94" spans="1:44" ht="13" customHeight="1">
       <c r="A94" s="102"/>
       <c r="B94" s="103"/>
       <c r="C94" s="103"/>
@@ -27325,7 +27325,7 @@
       <c r="AQ95" s="109"/>
       <c r="AR95" s="110"/>
     </row>
-    <row r="96" spans="1:44">
+    <row r="96" spans="1:44" ht="13" customHeight="1">
       <c r="A96" s="102"/>
       <c r="B96" s="103"/>
       <c r="C96" s="103"/>
@@ -27371,7 +27371,7 @@
       <c r="AQ96" s="109"/>
       <c r="AR96" s="110"/>
     </row>
-    <row r="97" spans="1:44">
+    <row r="97" spans="1:44" ht="13" customHeight="1">
       <c r="A97" s="102"/>
       <c r="B97" s="103"/>
       <c r="C97" s="103"/>
@@ -27417,7 +27417,7 @@
       <c r="AQ97" s="109"/>
       <c r="AR97" s="110"/>
     </row>
-    <row r="98" spans="1:44">
+    <row r="98" spans="1:44" ht="13" customHeight="1">
       <c r="A98" s="102"/>
       <c r="B98" s="103"/>
       <c r="C98" s="103"/>
@@ -27463,7 +27463,7 @@
       <c r="AQ98" s="109"/>
       <c r="AR98" s="110"/>
     </row>
-    <row r="99" spans="1:44">
+    <row r="99" spans="1:44" ht="13" customHeight="1">
       <c r="A99" s="102"/>
       <c r="B99" s="103"/>
       <c r="C99" s="103"/>
@@ -27511,7 +27511,7 @@
       <c r="AQ99" s="109"/>
       <c r="AR99" s="110"/>
     </row>
-    <row r="100" spans="1:44">
+    <row r="100" spans="1:44" ht="13" customHeight="1">
       <c r="A100" s="102"/>
       <c r="B100" s="103"/>
       <c r="C100" s="103"/>
@@ -27541,7 +27541,7 @@
       <c r="AQ100" s="109"/>
       <c r="AR100" s="110"/>
     </row>
-    <row r="101" spans="1:44">
+    <row r="101" spans="1:44" ht="13" customHeight="1">
       <c r="A101" s="102"/>
       <c r="B101" s="103"/>
       <c r="C101" s="103"/>
@@ -27571,7 +27571,7 @@
       <c r="AQ101" s="109"/>
       <c r="AR101" s="110"/>
     </row>
-    <row r="102" spans="1:44">
+    <row r="102" spans="1:44" ht="13" customHeight="1">
       <c r="A102" s="102"/>
       <c r="B102" s="103"/>
       <c r="C102" s="103"/>
@@ -27617,7 +27617,7 @@
       <c r="AQ102" s="109"/>
       <c r="AR102" s="110"/>
     </row>
-    <row r="103" spans="1:44" ht="15" thickBot="1">
+    <row r="103" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A103" s="117"/>
       <c r="B103" s="118"/>
       <c r="C103" s="118"/>
@@ -27715,7 +27715,7 @@
       <c r="AQ104" s="109"/>
       <c r="AR104" s="110"/>
     </row>
-    <row r="105" spans="1:44">
+    <row r="105" spans="1:44" ht="13" customHeight="1">
       <c r="A105" s="102"/>
       <c r="B105" s="103"/>
       <c r="C105" s="103"/>
@@ -27761,7 +27761,7 @@
       <c r="AQ105" s="109"/>
       <c r="AR105" s="110"/>
     </row>
-    <row r="106" spans="1:44">
+    <row r="106" spans="1:44" ht="13" customHeight="1">
       <c r="A106" s="102"/>
       <c r="B106" s="103"/>
       <c r="C106" s="103"/>
@@ -27807,7 +27807,7 @@
       <c r="AQ106" s="109"/>
       <c r="AR106" s="110"/>
     </row>
-    <row r="107" spans="1:44">
+    <row r="107" spans="1:44" ht="13" customHeight="1">
       <c r="A107" s="102"/>
       <c r="B107" s="103"/>
       <c r="C107" s="103"/>
@@ -27853,7 +27853,7 @@
       <c r="AQ107" s="109"/>
       <c r="AR107" s="110"/>
     </row>
-    <row r="108" spans="1:44" ht="15" thickBot="1">
+    <row r="108" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A108" s="117"/>
       <c r="B108" s="118"/>
       <c r="C108" s="118"/>
@@ -27899,7 +27899,7 @@
       <c r="AQ108" s="109"/>
       <c r="AR108" s="110"/>
     </row>
-    <row r="109" spans="1:44">
+    <row r="109" spans="1:44" ht="13" customHeight="1">
       <c r="A109" s="188" t="s">
         <v>220</v>
       </c>
@@ -27951,7 +27951,7 @@
       <c r="AQ109" s="109"/>
       <c r="AR109" s="110"/>
     </row>
-    <row r="110" spans="1:44">
+    <row r="110" spans="1:44" ht="13" customHeight="1">
       <c r="A110" s="151"/>
       <c r="B110" s="152"/>
       <c r="C110" s="152"/>
@@ -27997,7 +27997,7 @@
       <c r="AQ110" s="109"/>
       <c r="AR110" s="110"/>
     </row>
-    <row r="111" spans="1:44" ht="15" thickBot="1">
+    <row r="111" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A111" s="154"/>
       <c r="B111" s="155"/>
       <c r="C111" s="155"/>
@@ -28043,7 +28043,7 @@
       <c r="AQ111" s="109"/>
       <c r="AR111" s="110"/>
     </row>
-    <row r="112" spans="1:44">
+    <row r="112" spans="1:44" ht="13" customHeight="1">
       <c r="A112" s="99" t="s">
         <v>221</v>
       </c>
@@ -28095,7 +28095,7 @@
       <c r="AQ112" s="109"/>
       <c r="AR112" s="110"/>
     </row>
-    <row r="113" spans="1:44">
+    <row r="113" spans="1:44" ht="13" customHeight="1">
       <c r="A113" s="102"/>
       <c r="B113" s="103"/>
       <c r="C113" s="103"/>
@@ -28141,7 +28141,7 @@
       <c r="AQ113" s="109"/>
       <c r="AR113" s="110"/>
     </row>
-    <row r="114" spans="1:44" ht="15" thickBot="1">
+    <row r="114" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A114" s="102"/>
       <c r="B114" s="103"/>
       <c r="C114" s="103"/>
@@ -28283,7 +28283,7 @@
       <c r="AQ116" s="109"/>
       <c r="AR116" s="110"/>
     </row>
-    <row r="117" spans="1:44" ht="15" thickBot="1">
+    <row r="117" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A117" s="117"/>
       <c r="B117" s="118"/>
       <c r="C117" s="118"/>
@@ -28383,7 +28383,7 @@
       <c r="AQ118" s="106"/>
       <c r="AR118" s="107"/>
     </row>
-    <row r="119" spans="1:44">
+    <row r="119" spans="1:44" ht="13" customHeight="1">
       <c r="A119" s="151"/>
       <c r="B119" s="152"/>
       <c r="C119" s="152"/>
@@ -28429,7 +28429,7 @@
       <c r="AQ119" s="109"/>
       <c r="AR119" s="110"/>
     </row>
-    <row r="120" spans="1:44">
+    <row r="120" spans="1:44" ht="13" customHeight="1">
       <c r="A120" s="190"/>
       <c r="B120" s="191"/>
       <c r="C120" s="191"/>
@@ -28475,7 +28475,7 @@
       <c r="AQ120" s="109"/>
       <c r="AR120" s="110"/>
     </row>
-    <row r="121" spans="1:44" ht="7.5" customHeight="1" thickBot="1">
+    <row r="121" spans="1:44" thickBot="1" ht="7.5" customHeight="1">
       <c r="A121" s="190"/>
       <c r="B121" s="191"/>
       <c r="C121" s="191"/>
@@ -29217,7 +29217,7 @@
       <c r="AQ136" s="109"/>
       <c r="AR136" s="110"/>
     </row>
-    <row r="137" spans="1:44" ht="15" customHeight="1" thickBot="1">
+    <row r="137" spans="1:44" thickBot="1" ht="15" customHeight="1">
       <c r="A137" s="190"/>
       <c r="B137" s="191"/>
       <c r="C137" s="191"/>
@@ -29263,7 +29263,7 @@
       <c r="AQ137" s="109"/>
       <c r="AR137" s="110"/>
     </row>
-    <row r="138" spans="1:44">
+    <row r="138" spans="1:44" ht="13" customHeight="1">
       <c r="A138" s="188" t="s">
         <v>223</v>
       </c>
@@ -29315,7 +29315,7 @@
       <c r="AQ138" s="109"/>
       <c r="AR138" s="110"/>
     </row>
-    <row r="139" spans="1:44">
+    <row r="139" spans="1:44" ht="13" customHeight="1">
       <c r="A139" s="189"/>
       <c r="B139" s="169"/>
       <c r="C139" s="169"/>
@@ -29361,7 +29361,7 @@
       <c r="AQ139" s="109"/>
       <c r="AR139" s="110"/>
     </row>
-    <row r="140" spans="1:44">
+    <row r="140" spans="1:44" ht="13" customHeight="1">
       <c r="A140" s="189"/>
       <c r="B140" s="169"/>
       <c r="C140" s="169"/>
@@ -29407,7 +29407,7 @@
       <c r="AQ140" s="109"/>
       <c r="AR140" s="110"/>
     </row>
-    <row r="141" spans="1:44">
+    <row r="141" spans="1:44" ht="13" customHeight="1">
       <c r="A141" s="189"/>
       <c r="B141" s="169"/>
       <c r="C141" s="169"/>
@@ -29453,7 +29453,7 @@
       <c r="AQ141" s="109"/>
       <c r="AR141" s="110"/>
     </row>
-    <row r="142" spans="1:44">
+    <row r="142" spans="1:44" ht="13" customHeight="1">
       <c r="A142" s="151"/>
       <c r="B142" s="152"/>
       <c r="C142" s="152"/>
@@ -29499,7 +29499,7 @@
       <c r="AQ142" s="109"/>
       <c r="AR142" s="110"/>
     </row>
-    <row r="143" spans="1:44" ht="15" thickBot="1">
+    <row r="143" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A143" s="190"/>
       <c r="B143" s="191"/>
       <c r="C143" s="191"/>
@@ -29545,7 +29545,7 @@
       <c r="AQ143" s="109"/>
       <c r="AR143" s="110"/>
     </row>
-    <row r="144" spans="1:44">
+    <row r="144" spans="1:44" ht="13" customHeight="1">
       <c r="A144" s="188" t="s">
         <v>155</v>
       </c>
@@ -29597,7 +29597,7 @@
       <c r="AQ144" s="109"/>
       <c r="AR144" s="110"/>
     </row>
-    <row r="145" spans="1:44">
+    <row r="145" spans="1:44" ht="13" customHeight="1">
       <c r="A145" s="151"/>
       <c r="B145" s="152"/>
       <c r="C145" s="152"/>
@@ -29643,7 +29643,7 @@
       <c r="AQ145" s="109"/>
       <c r="AR145" s="110"/>
     </row>
-    <row r="146" spans="1:44">
+    <row r="146" spans="1:44" ht="13" customHeight="1">
       <c r="A146" s="190"/>
       <c r="B146" s="191"/>
       <c r="C146" s="191"/>
@@ -29689,7 +29689,7 @@
       <c r="AQ146" s="109"/>
       <c r="AR146" s="110"/>
     </row>
-    <row r="147" spans="1:44" ht="15" thickBot="1">
+    <row r="147" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A147" s="190"/>
       <c r="B147" s="191"/>
       <c r="C147" s="191"/>
@@ -29787,7 +29787,7 @@
       <c r="AQ148" s="106"/>
       <c r="AR148" s="107"/>
     </row>
-    <row r="149" spans="1:44">
+    <row r="149" spans="1:44" ht="13" customHeight="1">
       <c r="A149" s="102"/>
       <c r="B149" s="103"/>
       <c r="C149" s="103"/>
@@ -29833,7 +29833,7 @@
       <c r="AQ149" s="109"/>
       <c r="AR149" s="110"/>
     </row>
-    <row r="150" spans="1:44" ht="15" thickBot="1">
+    <row r="150" spans="1:44" thickBot="1" ht="13.5" customHeight="1">
       <c r="A150" s="102"/>
       <c r="B150" s="103"/>
       <c r="C150" s="103"/>
@@ -29879,7 +29879,7 @@
       <c r="AQ150" s="112"/>
       <c r="AR150" s="113"/>
     </row>
-    <row r="151" spans="1:44" ht="113.25" customHeight="1" thickBot="1">
+    <row r="151" spans="1:44" thickBot="1" ht="113.25" customHeight="1">
       <c r="A151" s="114" t="s">
         <v>249</v>
       </c>
@@ -29933,7 +29933,7 @@
       <c r="AQ151" s="239"/>
       <c r="AR151" s="240"/>
     </row>
-    <row r="152" spans="1:44">
+    <row r="152" spans="1:44" ht="13" customHeight="1">
       <c r="A152" s="38"/>
       <c r="B152" s="38"/>
       <c r="C152" s="38"/>
@@ -30081,17 +30081,17 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AL47"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="2.33203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="2.33203125" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col min="1" max="16384" width="2.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" ht="15" thickBot="1">
+    <row r="1" spans="1:38" thickBot="1" ht="12.5" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:38">
+    <row r="2" spans="1:38" ht="12" customHeight="1">
       <c r="A2" s="322" t="s">
         <v>30</v>
       </c>
@@ -30137,7 +30137,7 @@
       <c r="AK2" s="323"/>
       <c r="AL2" s="414"/>
     </row>
-    <row r="3" spans="1:38">
+    <row r="3" spans="1:38" ht="12" customHeight="1">
       <c r="A3" s="439"/>
       <c r="B3" s="440"/>
       <c r="C3" s="440"/>
@@ -30177,7 +30177,7 @@
       <c r="AK3" s="440"/>
       <c r="AL3" s="441"/>
     </row>
-    <row r="4" spans="1:38">
+    <row r="4" spans="1:38" ht="12" customHeight="1">
       <c r="A4" s="439" t="s">
         <v>29</v>
       </c>
@@ -30223,7 +30223,7 @@
       <c r="AK4" s="681"/>
       <c r="AL4" s="682"/>
     </row>
-    <row r="5" spans="1:38">
+    <row r="5" spans="1:38" ht="12" customHeight="1">
       <c r="A5" s="439"/>
       <c r="B5" s="440"/>
       <c r="C5" s="440"/>
@@ -30263,7 +30263,7 @@
       <c r="AK5" s="681"/>
       <c r="AL5" s="682"/>
     </row>
-    <row r="6" spans="1:38">
+    <row r="6" spans="1:38" ht="12" customHeight="1">
       <c r="A6" s="439"/>
       <c r="B6" s="440"/>
       <c r="C6" s="440"/>
@@ -30303,7 +30303,7 @@
       <c r="AK6" s="681"/>
       <c r="AL6" s="682"/>
     </row>
-    <row r="7" spans="1:38">
+    <row r="7" spans="1:38" ht="12" customHeight="1">
       <c r="A7" s="439"/>
       <c r="B7" s="440"/>
       <c r="C7" s="440"/>
@@ -30343,7 +30343,7 @@
       <c r="AK7" s="681"/>
       <c r="AL7" s="682"/>
     </row>
-    <row r="8" spans="1:38">
+    <row r="8" spans="1:38" ht="12" customHeight="1">
       <c r="A8" s="439" t="s">
         <v>32</v>
       </c>
@@ -30389,7 +30389,7 @@
       <c r="AK8" s="451"/>
       <c r="AL8" s="452"/>
     </row>
-    <row r="9" spans="1:38">
+    <row r="9" spans="1:38" ht="12" customHeight="1">
       <c r="A9" s="439"/>
       <c r="B9" s="440"/>
       <c r="C9" s="440"/>
@@ -30429,7 +30429,7 @@
       <c r="AK9" s="451"/>
       <c r="AL9" s="452"/>
     </row>
-    <row r="10" spans="1:38">
+    <row r="10" spans="1:38" ht="12" customHeight="1">
       <c r="A10" s="439"/>
       <c r="B10" s="440"/>
       <c r="C10" s="440"/>
@@ -30469,7 +30469,7 @@
       <c r="AK10" s="451"/>
       <c r="AL10" s="452"/>
     </row>
-    <row r="11" spans="1:38">
+    <row r="11" spans="1:38" ht="12" customHeight="1">
       <c r="A11" s="439"/>
       <c r="B11" s="440"/>
       <c r="C11" s="440"/>
@@ -30509,7 +30509,7 @@
       <c r="AK11" s="451"/>
       <c r="AL11" s="452"/>
     </row>
-    <row r="12" spans="1:38">
+    <row r="12" spans="1:38" ht="12" customHeight="1">
       <c r="A12" s="439" t="s">
         <v>36</v>
       </c>
@@ -30555,7 +30555,7 @@
       <c r="AK12" s="451"/>
       <c r="AL12" s="452"/>
     </row>
-    <row r="13" spans="1:38">
+    <row r="13" spans="1:38" ht="12" customHeight="1">
       <c r="A13" s="439"/>
       <c r="B13" s="440"/>
       <c r="C13" s="440"/>
@@ -30595,7 +30595,7 @@
       <c r="AK13" s="451"/>
       <c r="AL13" s="452"/>
     </row>
-    <row r="14" spans="1:38">
+    <row r="14" spans="1:38" ht="12" customHeight="1">
       <c r="A14" s="439"/>
       <c r="B14" s="440"/>
       <c r="C14" s="440"/>
@@ -30635,7 +30635,7 @@
       <c r="AK14" s="451"/>
       <c r="AL14" s="452"/>
     </row>
-    <row r="15" spans="1:38">
+    <row r="15" spans="1:38" ht="12" customHeight="1">
       <c r="A15" s="439"/>
       <c r="B15" s="440"/>
       <c r="C15" s="440"/>
@@ -30675,7 +30675,7 @@
       <c r="AK15" s="451"/>
       <c r="AL15" s="452"/>
     </row>
-    <row r="16" spans="1:38">
+    <row r="16" spans="1:38" ht="12" customHeight="1">
       <c r="A16" s="439" t="s">
         <v>40</v>
       </c>
@@ -30721,7 +30721,7 @@
       <c r="AK16" s="451"/>
       <c r="AL16" s="452"/>
     </row>
-    <row r="17" spans="1:38">
+    <row r="17" spans="1:38" ht="12" customHeight="1">
       <c r="A17" s="439"/>
       <c r="B17" s="440"/>
       <c r="C17" s="440"/>
@@ -30761,7 +30761,7 @@
       <c r="AK17" s="451"/>
       <c r="AL17" s="452"/>
     </row>
-    <row r="18" spans="1:38">
+    <row r="18" spans="1:38" ht="12" customHeight="1">
       <c r="A18" s="439"/>
       <c r="B18" s="440"/>
       <c r="C18" s="440"/>
@@ -30801,7 +30801,7 @@
       <c r="AK18" s="451"/>
       <c r="AL18" s="452"/>
     </row>
-    <row r="19" spans="1:38" ht="15" thickBot="1">
+    <row r="19" spans="1:38" thickBot="1" ht="12.5" customHeight="1">
       <c r="A19" s="325"/>
       <c r="B19" s="326"/>
       <c r="C19" s="326"/>
@@ -30841,17 +30841,17 @@
       <c r="AK19" s="453"/>
       <c r="AL19" s="454"/>
     </row>
-    <row r="20" spans="1:38">
+    <row r="20" spans="1:38" ht="12" customHeight="1">
       <c r="A20" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:38" ht="15" thickBot="1">
+    <row r="23" spans="1:38" thickBot="1" ht="12.5" customHeight="1">
       <c r="A23" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="24" spans="1:38">
+    <row r="24" spans="1:38" ht="12" customHeight="1">
       <c r="A24" s="322" t="s">
         <v>29</v>
       </c>
@@ -30895,7 +30895,7 @@
       <c r="AK24" s="544"/>
       <c r="AL24" s="545"/>
     </row>
-    <row r="25" spans="1:38">
+    <row r="25" spans="1:38" ht="12" customHeight="1">
       <c r="A25" s="439"/>
       <c r="B25" s="440"/>
       <c r="C25" s="440"/>
@@ -30935,7 +30935,7 @@
       <c r="AK25" s="451"/>
       <c r="AL25" s="452"/>
     </row>
-    <row r="26" spans="1:38">
+    <row r="26" spans="1:38" ht="12" customHeight="1">
       <c r="A26" s="439" t="s">
         <v>32</v>
       </c>
@@ -30979,7 +30979,7 @@
       <c r="AK26" s="451"/>
       <c r="AL26" s="452"/>
     </row>
-    <row r="27" spans="1:38">
+    <row r="27" spans="1:38" ht="12" customHeight="1">
       <c r="A27" s="439"/>
       <c r="B27" s="440"/>
       <c r="C27" s="440"/>
@@ -31019,7 +31019,7 @@
       <c r="AK27" s="451"/>
       <c r="AL27" s="452"/>
     </row>
-    <row r="28" spans="1:38">
+    <row r="28" spans="1:38" ht="12" customHeight="1">
       <c r="A28" s="439" t="s">
         <v>36</v>
       </c>
@@ -31063,7 +31063,7 @@
       <c r="AK28" s="451"/>
       <c r="AL28" s="452"/>
     </row>
-    <row r="29" spans="1:38">
+    <row r="29" spans="1:38" ht="12" customHeight="1">
       <c r="A29" s="439"/>
       <c r="B29" s="440"/>
       <c r="C29" s="440"/>
@@ -31103,7 +31103,7 @@
       <c r="AK29" s="451"/>
       <c r="AL29" s="452"/>
     </row>
-    <row r="30" spans="1:38">
+    <row r="30" spans="1:38" ht="12" customHeight="1">
       <c r="A30" s="439"/>
       <c r="B30" s="440"/>
       <c r="C30" s="440"/>
@@ -31145,7 +31145,7 @@
       <c r="AK30" s="451"/>
       <c r="AL30" s="452"/>
     </row>
-    <row r="31" spans="1:38">
+    <row r="31" spans="1:38" ht="12" customHeight="1">
       <c r="A31" s="439"/>
       <c r="B31" s="440"/>
       <c r="C31" s="440"/>
@@ -31185,7 +31185,7 @@
       <c r="AK31" s="451"/>
       <c r="AL31" s="452"/>
     </row>
-    <row r="32" spans="1:38">
+    <row r="32" spans="1:38" ht="12" customHeight="1">
       <c r="A32" s="439" t="s">
         <v>54</v>
       </c>
@@ -31229,7 +31229,7 @@
       <c r="AK32" s="681"/>
       <c r="AL32" s="682"/>
     </row>
-    <row r="33" spans="1:38">
+    <row r="33" spans="1:38" ht="12" customHeight="1">
       <c r="A33" s="439"/>
       <c r="B33" s="440"/>
       <c r="C33" s="440"/>
@@ -31269,7 +31269,7 @@
       <c r="AK33" s="681"/>
       <c r="AL33" s="682"/>
     </row>
-    <row r="34" spans="1:38">
+    <row r="34" spans="1:38" ht="12" customHeight="1">
       <c r="A34" s="439"/>
       <c r="B34" s="440"/>
       <c r="C34" s="440"/>
@@ -31309,7 +31309,7 @@
       <c r="AK34" s="681"/>
       <c r="AL34" s="682"/>
     </row>
-    <row r="35" spans="1:38">
+    <row r="35" spans="1:38" ht="12" customHeight="1">
       <c r="A35" s="439"/>
       <c r="B35" s="440"/>
       <c r="C35" s="440"/>
@@ -31349,7 +31349,7 @@
       <c r="AK35" s="681"/>
       <c r="AL35" s="682"/>
     </row>
-    <row r="36" spans="1:38">
+    <row r="36" spans="1:38" ht="12" customHeight="1">
       <c r="A36" s="439"/>
       <c r="B36" s="440"/>
       <c r="C36" s="440"/>
@@ -31391,7 +31391,7 @@
       <c r="AK36" s="451"/>
       <c r="AL36" s="452"/>
     </row>
-    <row r="37" spans="1:38">
+    <row r="37" spans="1:38" ht="12" customHeight="1">
       <c r="A37" s="439"/>
       <c r="B37" s="440"/>
       <c r="C37" s="440"/>
@@ -31431,7 +31431,7 @@
       <c r="AK37" s="451"/>
       <c r="AL37" s="452"/>
     </row>
-    <row r="38" spans="1:38">
+    <row r="38" spans="1:38" ht="12" customHeight="1">
       <c r="A38" s="439"/>
       <c r="B38" s="440"/>
       <c r="C38" s="440"/>
@@ -31473,7 +31473,7 @@
       <c r="AK38" s="451"/>
       <c r="AL38" s="452"/>
     </row>
-    <row r="39" spans="1:38">
+    <row r="39" spans="1:38" ht="12" customHeight="1">
       <c r="A39" s="439"/>
       <c r="B39" s="440"/>
       <c r="C39" s="440"/>
@@ -31513,7 +31513,7 @@
       <c r="AK39" s="451"/>
       <c r="AL39" s="452"/>
     </row>
-    <row r="40" spans="1:38">
+    <row r="40" spans="1:38" ht="12" customHeight="1">
       <c r="A40" s="439"/>
       <c r="B40" s="440"/>
       <c r="C40" s="440"/>
@@ -31555,7 +31555,7 @@
       <c r="AK40" s="451"/>
       <c r="AL40" s="452"/>
     </row>
-    <row r="41" spans="1:38">
+    <row r="41" spans="1:38" ht="12" customHeight="1">
       <c r="A41" s="439"/>
       <c r="B41" s="440"/>
       <c r="C41" s="440"/>
@@ -31595,7 +31595,7 @@
       <c r="AK41" s="451"/>
       <c r="AL41" s="452"/>
     </row>
-    <row r="42" spans="1:38">
+    <row r="42" spans="1:38" ht="12" customHeight="1">
       <c r="A42" s="439"/>
       <c r="B42" s="440"/>
       <c r="C42" s="440"/>
@@ -31637,7 +31637,7 @@
       <c r="AK42" s="451"/>
       <c r="AL42" s="452"/>
     </row>
-    <row r="43" spans="1:38">
+    <row r="43" spans="1:38" ht="12" customHeight="1">
       <c r="A43" s="439"/>
       <c r="B43" s="440"/>
       <c r="C43" s="440"/>
@@ -31677,7 +31677,7 @@
       <c r="AK43" s="451"/>
       <c r="AL43" s="452"/>
     </row>
-    <row r="44" spans="1:38">
+    <row r="44" spans="1:38" ht="12" customHeight="1">
       <c r="A44" s="439"/>
       <c r="B44" s="440"/>
       <c r="C44" s="440"/>
@@ -31719,7 +31719,7 @@
       <c r="AK44" s="451"/>
       <c r="AL44" s="452"/>
     </row>
-    <row r="45" spans="1:38">
+    <row r="45" spans="1:38" ht="12" customHeight="1">
       <c r="A45" s="439"/>
       <c r="B45" s="440"/>
       <c r="C45" s="440"/>
@@ -31759,7 +31759,7 @@
       <c r="AK45" s="451"/>
       <c r="AL45" s="452"/>
     </row>
-    <row r="46" spans="1:38">
+    <row r="46" spans="1:38" ht="12" customHeight="1">
       <c r="A46" s="439"/>
       <c r="B46" s="440"/>
       <c r="C46" s="440"/>
@@ -31801,7 +31801,7 @@
       <c r="AK46" s="451"/>
       <c r="AL46" s="452"/>
     </row>
-    <row r="47" spans="1:38" ht="15" thickBot="1">
+    <row r="47" spans="1:38" thickBot="1" ht="12.5" customHeight="1">
       <c r="A47" s="325"/>
       <c r="B47" s="326"/>
       <c r="C47" s="326"/>

</xml_diff>